<commit_message>
journals and reports 25.09.2026
</commit_message>
<xml_diff>
--- a/ჟურნალი/4. N301 front-end დეველოპმენტი (ინტეგრირებული მიდგომით) - TypeScript.xlsx
+++ b/ჟურნალი/4. N301 front-end დეველოპმენტი (ინტეგრირებული მიდგომით) - TypeScript.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3Daudiece\Desktop\Front-end!!\0. ready\ჟურნალი\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\designer\Desktop\Front\01. - Front-end-docs\ჟურნალი\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8A0702-49D6-4E98-B8B6-2CBA26E2BE0E}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8A0702-49D6-4E98-B8B6-2CBA26E2BE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="367" yWindow="14" windowWidth="20962" windowHeight="9727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="301 ინტეგრირებული" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -769,7 +782,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -807,23 +820,113 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -855,9 +958,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -875,99 +975,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="7" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1186,145 +1193,145 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:ET31"/>
-  <sheetFormatPr defaultColWidth="3.625" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="3.5703125" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.625" style="2"/>
+    <col min="1" max="1" width="3.5703125" style="2"/>
     <col min="2" max="3" width="21" style="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="1" customWidth="1"/>
-    <col min="5" max="5" width="5.625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="3.625" style="1"/>
+    <col min="5" max="5" width="5.5703125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="3.5703125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="27" t="s">
+      <c r="A1" s="56" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="28"/>
-      <c r="F1" s="31">
+      <c r="C1" s="57"/>
+      <c r="D1" s="58"/>
+      <c r="F1" s="61">
         <v>4</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="33">
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="32">
         <v>3</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33">
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32">
         <v>4</v>
       </c>
-      <c r="N1" s="33"/>
-      <c r="O1" s="33"/>
-      <c r="P1" s="33"/>
-      <c r="Q1" s="34">
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="63">
         <v>4</v>
       </c>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="36"/>
-      <c r="U1" s="34">
+      <c r="R1" s="64"/>
+      <c r="S1" s="64"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="63">
         <v>4</v>
       </c>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="36"/>
-      <c r="Y1" s="34">
+      <c r="V1" s="64"/>
+      <c r="W1" s="64"/>
+      <c r="X1" s="65"/>
+      <c r="Y1" s="63">
         <v>4</v>
       </c>
-      <c r="Z1" s="35"/>
-      <c r="AA1" s="35"/>
-      <c r="AB1" s="36"/>
-      <c r="AC1" s="66">
+      <c r="Z1" s="64"/>
+      <c r="AA1" s="64"/>
+      <c r="AB1" s="65"/>
+      <c r="AC1" s="30">
         <v>2</v>
       </c>
-      <c r="AD1" s="67"/>
-      <c r="AE1" s="44">
+      <c r="AD1" s="31"/>
+      <c r="AE1" s="21">
         <v>4</v>
       </c>
-      <c r="AF1" s="45"/>
-      <c r="AG1" s="45"/>
-      <c r="AH1" s="46"/>
-      <c r="AI1" s="44">
+      <c r="AF1" s="22"/>
+      <c r="AG1" s="22"/>
+      <c r="AH1" s="23"/>
+      <c r="AI1" s="21">
         <v>4</v>
       </c>
-      <c r="AJ1" s="45"/>
-      <c r="AK1" s="45"/>
-      <c r="AL1" s="46"/>
-      <c r="AM1" s="44">
+      <c r="AJ1" s="22"/>
+      <c r="AK1" s="22"/>
+      <c r="AL1" s="23"/>
+      <c r="AM1" s="21">
         <v>2</v>
       </c>
-      <c r="AN1" s="46"/>
-      <c r="AO1" s="44">
+      <c r="AN1" s="23"/>
+      <c r="AO1" s="21">
         <v>4</v>
       </c>
-      <c r="AP1" s="45"/>
-      <c r="AQ1" s="45"/>
-      <c r="AR1" s="46"/>
-      <c r="AS1" s="44">
+      <c r="AP1" s="22"/>
+      <c r="AQ1" s="22"/>
+      <c r="AR1" s="23"/>
+      <c r="AS1" s="21">
         <v>5</v>
       </c>
-      <c r="AT1" s="45"/>
-      <c r="AU1" s="45"/>
-      <c r="AV1" s="45"/>
-      <c r="AW1" s="46"/>
+      <c r="AT1" s="22"/>
+      <c r="AU1" s="22"/>
+      <c r="AV1" s="22"/>
+      <c r="AW1" s="23"/>
       <c r="AX1" s="3">
         <v>1</v>
       </c>
-      <c r="AY1" s="44">
+      <c r="AY1" s="21">
         <v>5</v>
       </c>
-      <c r="AZ1" s="45"/>
-      <c r="BA1" s="45"/>
-      <c r="BB1" s="45"/>
-      <c r="BC1" s="46"/>
-      <c r="BD1" s="44">
+      <c r="AZ1" s="22"/>
+      <c r="BA1" s="22"/>
+      <c r="BB1" s="22"/>
+      <c r="BC1" s="23"/>
+      <c r="BD1" s="21">
         <v>3</v>
       </c>
-      <c r="BE1" s="45"/>
-      <c r="BF1" s="46"/>
-      <c r="BG1" s="20">
+      <c r="BE1" s="22"/>
+      <c r="BF1" s="23"/>
+      <c r="BG1" s="3">
         <v>1</v>
       </c>
-      <c r="BH1" s="33">
+      <c r="BH1" s="32">
         <v>5</v>
       </c>
-      <c r="BI1" s="33"/>
-      <c r="BJ1" s="33"/>
-      <c r="BK1" s="33"/>
-      <c r="BL1" s="33"/>
-      <c r="BM1" s="44">
+      <c r="BI1" s="32"/>
+      <c r="BJ1" s="32"/>
+      <c r="BK1" s="32"/>
+      <c r="BL1" s="32"/>
+      <c r="BM1" s="21">
         <v>3</v>
       </c>
-      <c r="BN1" s="45"/>
-      <c r="BO1" s="46"/>
-      <c r="BP1" s="21">
+      <c r="BN1" s="22"/>
+      <c r="BO1" s="23"/>
+      <c r="BP1" s="20">
         <v>1</v>
       </c>
-      <c r="BQ1" s="68">
+      <c r="BQ1" s="24">
         <v>5</v>
       </c>
-      <c r="BR1" s="69"/>
-      <c r="BS1" s="69"/>
-      <c r="BT1" s="69"/>
-      <c r="BU1" s="70"/>
-      <c r="BV1" s="44">
+      <c r="BR1" s="25"/>
+      <c r="BS1" s="25"/>
+      <c r="BT1" s="25"/>
+      <c r="BU1" s="26"/>
+      <c r="BV1" s="21">
         <v>3</v>
       </c>
-      <c r="BW1" s="45"/>
-      <c r="BX1" s="46"/>
-      <c r="BY1" s="22">
+      <c r="BW1" s="22"/>
+      <c r="BX1" s="23"/>
+      <c r="BY1" s="3">
         <v>1</v>
       </c>
-      <c r="BZ1" s="44">
+      <c r="BZ1" s="21">
         <v>3</v>
       </c>
-      <c r="CA1" s="45"/>
-      <c r="CB1" s="46"/>
+      <c r="CA1" s="22"/>
+      <c r="CB1" s="23"/>
       <c r="CC1" s="4"/>
       <c r="CD1" s="4"/>
       <c r="CE1" s="4"/>
@@ -1396,1644 +1403,1644 @@
       </c>
     </row>
     <row r="2" spans="1:150" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="37" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="F2" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="42" t="s">
+      <c r="G2" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="H2" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="42" t="s">
+      <c r="I2" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="40" t="s">
+      <c r="J2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="42" t="s">
+      <c r="K2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="42" t="s">
+      <c r="L2" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="40" t="s">
+      <c r="M2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="40" t="s">
+      <c r="N2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="O2" s="40" t="s">
+      <c r="O2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="P2" s="40" t="s">
+      <c r="P2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="Q2" s="40" t="s">
+      <c r="Q2" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="R2" s="42" t="s">
+      <c r="R2" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="S2" s="42" t="s">
+      <c r="S2" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="T2" s="42" t="s">
+      <c r="T2" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="U2" s="40" t="s">
+      <c r="U2" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="V2" s="42" t="s">
+      <c r="V2" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="W2" s="42" t="s">
+      <c r="W2" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="X2" s="42" t="s">
+      <c r="X2" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="Y2" s="40" t="s">
+      <c r="Y2" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="Z2" s="42" t="s">
+      <c r="Z2" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="AA2" s="47" t="s">
+      <c r="AA2" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="AB2" s="47" t="s">
+      <c r="AB2" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="AC2" s="40">
+      <c r="AC2" s="39">
         <v>46199</v>
       </c>
-      <c r="AD2" s="40">
+      <c r="AD2" s="39">
         <v>46199</v>
       </c>
-      <c r="AE2" s="40">
+      <c r="AE2" s="39">
         <v>46202</v>
       </c>
-      <c r="AF2" s="40">
+      <c r="AF2" s="39">
         <v>46202</v>
       </c>
-      <c r="AG2" s="40">
+      <c r="AG2" s="39">
         <v>46202</v>
       </c>
-      <c r="AH2" s="40">
+      <c r="AH2" s="39">
         <v>46202</v>
       </c>
-      <c r="AI2" s="40">
+      <c r="AI2" s="39">
         <v>46205</v>
       </c>
-      <c r="AJ2" s="40">
+      <c r="AJ2" s="39">
         <v>46205</v>
       </c>
-      <c r="AK2" s="40">
+      <c r="AK2" s="39">
         <v>46205</v>
       </c>
-      <c r="AL2" s="40">
+      <c r="AL2" s="39">
         <v>46205</v>
       </c>
-      <c r="AM2" s="40">
+      <c r="AM2" s="39">
         <v>46206</v>
       </c>
-      <c r="AN2" s="40">
+      <c r="AN2" s="39">
         <v>46206</v>
       </c>
-      <c r="AO2" s="40">
+      <c r="AO2" s="39">
         <v>46212</v>
       </c>
-      <c r="AP2" s="40">
+      <c r="AP2" s="39">
         <v>46212</v>
       </c>
-      <c r="AQ2" s="40">
+      <c r="AQ2" s="39">
         <v>46212</v>
       </c>
-      <c r="AR2" s="40">
+      <c r="AR2" s="39">
         <v>46212</v>
       </c>
-      <c r="AS2" s="40">
+      <c r="AS2" s="39">
         <v>46213</v>
       </c>
-      <c r="AT2" s="40">
+      <c r="AT2" s="39">
         <v>46213</v>
       </c>
-      <c r="AU2" s="40">
+      <c r="AU2" s="39">
         <v>46213</v>
       </c>
-      <c r="AV2" s="40">
+      <c r="AV2" s="39">
         <v>46213</v>
       </c>
-      <c r="AW2" s="40">
+      <c r="AW2" s="39">
         <v>46213</v>
       </c>
-      <c r="AX2" s="40">
+      <c r="AX2" s="39">
         <v>46218</v>
       </c>
-      <c r="AY2" s="40">
+      <c r="AY2" s="39">
         <v>46219</v>
       </c>
-      <c r="AZ2" s="40">
+      <c r="AZ2" s="39">
         <v>46219</v>
       </c>
-      <c r="BA2" s="40">
+      <c r="BA2" s="39">
         <v>46219</v>
       </c>
-      <c r="BB2" s="40">
+      <c r="BB2" s="39">
         <v>46219</v>
       </c>
-      <c r="BC2" s="40">
+      <c r="BC2" s="39">
         <v>46219</v>
       </c>
-      <c r="BD2" s="40">
+      <c r="BD2" s="39">
         <v>46220</v>
       </c>
-      <c r="BE2" s="40">
+      <c r="BE2" s="39">
         <v>46220</v>
       </c>
-      <c r="BF2" s="40">
+      <c r="BF2" s="39">
         <v>46220</v>
       </c>
-      <c r="BG2" s="40">
+      <c r="BG2" s="39">
         <v>46225</v>
       </c>
-      <c r="BH2" s="40">
+      <c r="BH2" s="39">
         <v>46226</v>
       </c>
-      <c r="BI2" s="40">
+      <c r="BI2" s="39">
         <v>46226</v>
       </c>
-      <c r="BJ2" s="40">
+      <c r="BJ2" s="39">
         <v>46226</v>
       </c>
-      <c r="BK2" s="40">
+      <c r="BK2" s="39">
         <v>46226</v>
       </c>
-      <c r="BL2" s="40">
+      <c r="BL2" s="39">
         <v>46226</v>
       </c>
-      <c r="BM2" s="40">
+      <c r="BM2" s="39">
         <v>46227</v>
       </c>
-      <c r="BN2" s="40">
+      <c r="BN2" s="39">
         <v>46227</v>
       </c>
-      <c r="BO2" s="40">
+      <c r="BO2" s="39">
         <v>46227</v>
       </c>
-      <c r="BP2" s="40">
+      <c r="BP2" s="39">
         <v>46232</v>
       </c>
-      <c r="BQ2" s="40">
+      <c r="BQ2" s="39">
         <v>46233</v>
       </c>
-      <c r="BR2" s="40">
+      <c r="BR2" s="39">
         <v>46233</v>
       </c>
-      <c r="BS2" s="40">
+      <c r="BS2" s="39">
         <v>46233</v>
       </c>
-      <c r="BT2" s="40">
+      <c r="BT2" s="39">
         <v>46233</v>
       </c>
-      <c r="BU2" s="40">
+      <c r="BU2" s="39">
         <v>46233</v>
       </c>
-      <c r="BV2" s="40">
+      <c r="BV2" s="39">
         <v>46234</v>
       </c>
-      <c r="BW2" s="40">
+      <c r="BW2" s="39">
         <v>46234</v>
       </c>
-      <c r="BX2" s="49">
+      <c r="BX2" s="47">
         <v>46234</v>
       </c>
-      <c r="BY2" s="40">
+      <c r="BY2" s="39">
         <v>46274</v>
       </c>
-      <c r="BZ2" s="40">
+      <c r="BZ2" s="39">
         <v>46276</v>
       </c>
-      <c r="CA2" s="40">
+      <c r="CA2" s="39">
         <v>46276</v>
       </c>
-      <c r="CB2" s="40">
+      <c r="CB2" s="39">
         <v>46276</v>
       </c>
-      <c r="CC2" s="40"/>
-      <c r="CD2" s="40"/>
-      <c r="CE2" s="40"/>
-      <c r="CF2" s="40"/>
-      <c r="CG2" s="40"/>
-      <c r="CH2" s="40"/>
-      <c r="CI2" s="40"/>
-      <c r="CJ2" s="40"/>
-      <c r="CK2" s="40"/>
-      <c r="CL2" s="40"/>
-      <c r="CM2" s="40"/>
-      <c r="CN2" s="40"/>
-      <c r="CO2" s="40"/>
-      <c r="CP2" s="40"/>
-      <c r="CQ2" s="40"/>
-      <c r="CR2" s="40"/>
-      <c r="CS2" s="40"/>
-      <c r="CT2" s="40"/>
-      <c r="CU2" s="40"/>
-      <c r="CV2" s="40"/>
-      <c r="CW2" s="40"/>
-      <c r="CX2" s="40"/>
-      <c r="CY2" s="40"/>
-      <c r="CZ2" s="40"/>
-      <c r="DA2" s="40"/>
-      <c r="DB2" s="40"/>
-      <c r="DC2" s="40"/>
-      <c r="DD2" s="40"/>
-      <c r="DE2" s="40"/>
-      <c r="DF2" s="40"/>
-      <c r="DG2" s="40"/>
-      <c r="DH2" s="40"/>
-      <c r="DI2" s="40"/>
-      <c r="DJ2" s="40"/>
-      <c r="DK2" s="40"/>
-      <c r="DL2" s="40"/>
-      <c r="DM2" s="40"/>
-      <c r="DN2" s="40"/>
-      <c r="DO2" s="40"/>
-      <c r="DP2" s="40"/>
-      <c r="DQ2" s="40"/>
-      <c r="DR2" s="40"/>
-      <c r="DS2" s="40"/>
-      <c r="DT2" s="40"/>
-      <c r="DU2" s="40"/>
-      <c r="DV2" s="40"/>
-      <c r="DW2" s="40"/>
-      <c r="DX2" s="40"/>
-      <c r="DY2" s="40"/>
-      <c r="DZ2" s="40"/>
-      <c r="EA2" s="40"/>
-      <c r="EB2" s="40"/>
-      <c r="EC2" s="40"/>
-      <c r="ED2" s="40"/>
-      <c r="EE2" s="40"/>
-      <c r="EF2" s="40"/>
-      <c r="EG2" s="40"/>
-      <c r="EH2" s="40"/>
-      <c r="EI2" s="40"/>
-      <c r="EJ2" s="40"/>
-      <c r="EK2" s="40"/>
-      <c r="EL2" s="40"/>
-      <c r="EM2" s="40"/>
-      <c r="EN2" s="40"/>
-      <c r="EO2" s="40"/>
+      <c r="CC2" s="39"/>
+      <c r="CD2" s="39"/>
+      <c r="CE2" s="39"/>
+      <c r="CF2" s="39"/>
+      <c r="CG2" s="39"/>
+      <c r="CH2" s="39"/>
+      <c r="CI2" s="39"/>
+      <c r="CJ2" s="39"/>
+      <c r="CK2" s="39"/>
+      <c r="CL2" s="39"/>
+      <c r="CM2" s="39"/>
+      <c r="CN2" s="39"/>
+      <c r="CO2" s="39"/>
+      <c r="CP2" s="39"/>
+      <c r="CQ2" s="39"/>
+      <c r="CR2" s="39"/>
+      <c r="CS2" s="39"/>
+      <c r="CT2" s="39"/>
+      <c r="CU2" s="39"/>
+      <c r="CV2" s="39"/>
+      <c r="CW2" s="39"/>
+      <c r="CX2" s="39"/>
+      <c r="CY2" s="39"/>
+      <c r="CZ2" s="39"/>
+      <c r="DA2" s="39"/>
+      <c r="DB2" s="39"/>
+      <c r="DC2" s="39"/>
+      <c r="DD2" s="39"/>
+      <c r="DE2" s="39"/>
+      <c r="DF2" s="39"/>
+      <c r="DG2" s="39"/>
+      <c r="DH2" s="39"/>
+      <c r="DI2" s="39"/>
+      <c r="DJ2" s="39"/>
+      <c r="DK2" s="39"/>
+      <c r="DL2" s="39"/>
+      <c r="DM2" s="39"/>
+      <c r="DN2" s="39"/>
+      <c r="DO2" s="39"/>
+      <c r="DP2" s="39"/>
+      <c r="DQ2" s="39"/>
+      <c r="DR2" s="39"/>
+      <c r="DS2" s="39"/>
+      <c r="DT2" s="39"/>
+      <c r="DU2" s="39"/>
+      <c r="DV2" s="39"/>
+      <c r="DW2" s="39"/>
+      <c r="DX2" s="39"/>
+      <c r="DY2" s="39"/>
+      <c r="DZ2" s="39"/>
+      <c r="EA2" s="39"/>
+      <c r="EB2" s="39"/>
+      <c r="EC2" s="39"/>
+      <c r="ED2" s="39"/>
+      <c r="EE2" s="39"/>
+      <c r="EF2" s="39"/>
+      <c r="EG2" s="39"/>
+      <c r="EH2" s="39"/>
+      <c r="EI2" s="39"/>
+      <c r="EJ2" s="39"/>
+      <c r="EK2" s="39"/>
+      <c r="EL2" s="39"/>
+      <c r="EM2" s="39"/>
+      <c r="EN2" s="39"/>
+      <c r="EO2" s="39"/>
     </row>
-    <row r="3" spans="1:150" ht="23.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="51" t="s">
+    <row r="3" spans="1:150" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="42"/>
-      <c r="S3" s="42"/>
-      <c r="T3" s="42"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="42"/>
-      <c r="W3" s="42"/>
-      <c r="X3" s="42"/>
-      <c r="Y3" s="40"/>
-      <c r="Z3" s="42"/>
-      <c r="AA3" s="47"/>
-      <c r="AB3" s="47"/>
-      <c r="AC3" s="40"/>
-      <c r="AD3" s="40"/>
-      <c r="AE3" s="40"/>
-      <c r="AF3" s="40"/>
-      <c r="AG3" s="40"/>
-      <c r="AH3" s="40"/>
-      <c r="AI3" s="40"/>
-      <c r="AJ3" s="40"/>
-      <c r="AK3" s="40"/>
-      <c r="AL3" s="40"/>
-      <c r="AM3" s="40"/>
-      <c r="AN3" s="40"/>
-      <c r="AO3" s="40"/>
-      <c r="AP3" s="40"/>
-      <c r="AQ3" s="40"/>
-      <c r="AR3" s="40"/>
-      <c r="AS3" s="40"/>
-      <c r="AT3" s="40"/>
-      <c r="AU3" s="40"/>
-      <c r="AV3" s="40"/>
-      <c r="AW3" s="40"/>
-      <c r="AX3" s="40"/>
-      <c r="AY3" s="40"/>
-      <c r="AZ3" s="40"/>
-      <c r="BA3" s="40"/>
-      <c r="BB3" s="40"/>
-      <c r="BC3" s="40"/>
-      <c r="BD3" s="40"/>
-      <c r="BE3" s="40"/>
-      <c r="BF3" s="40"/>
-      <c r="BG3" s="40"/>
-      <c r="BH3" s="40"/>
-      <c r="BI3" s="40"/>
-      <c r="BJ3" s="40"/>
-      <c r="BK3" s="40"/>
-      <c r="BL3" s="40"/>
-      <c r="BM3" s="40"/>
-      <c r="BN3" s="40"/>
-      <c r="BO3" s="40"/>
-      <c r="BP3" s="40"/>
-      <c r="BQ3" s="40"/>
-      <c r="BR3" s="40"/>
-      <c r="BS3" s="40"/>
-      <c r="BT3" s="40"/>
-      <c r="BU3" s="40"/>
-      <c r="BV3" s="40"/>
-      <c r="BW3" s="40"/>
-      <c r="BX3" s="49"/>
-      <c r="BY3" s="40"/>
-      <c r="BZ3" s="40"/>
-      <c r="CA3" s="40"/>
-      <c r="CB3" s="40"/>
-      <c r="CC3" s="40"/>
-      <c r="CD3" s="40"/>
-      <c r="CE3" s="40"/>
-      <c r="CF3" s="40"/>
-      <c r="CG3" s="40"/>
-      <c r="CH3" s="40"/>
-      <c r="CI3" s="40"/>
-      <c r="CJ3" s="40"/>
-      <c r="CK3" s="40"/>
-      <c r="CL3" s="40"/>
-      <c r="CM3" s="40"/>
-      <c r="CN3" s="40"/>
-      <c r="CO3" s="40"/>
-      <c r="CP3" s="40"/>
-      <c r="CQ3" s="40"/>
-      <c r="CR3" s="40"/>
-      <c r="CS3" s="40"/>
-      <c r="CT3" s="40"/>
-      <c r="CU3" s="40"/>
-      <c r="CV3" s="40"/>
-      <c r="CW3" s="40"/>
-      <c r="CX3" s="40"/>
-      <c r="CY3" s="40"/>
-      <c r="CZ3" s="40"/>
-      <c r="DA3" s="40"/>
-      <c r="DB3" s="40"/>
-      <c r="DC3" s="40"/>
-      <c r="DD3" s="40"/>
-      <c r="DE3" s="40"/>
-      <c r="DF3" s="40"/>
-      <c r="DG3" s="40"/>
-      <c r="DH3" s="40"/>
-      <c r="DI3" s="40"/>
-      <c r="DJ3" s="40"/>
-      <c r="DK3" s="40"/>
-      <c r="DL3" s="40"/>
-      <c r="DM3" s="40"/>
-      <c r="DN3" s="40"/>
-      <c r="DO3" s="40"/>
-      <c r="DP3" s="40"/>
-      <c r="DQ3" s="40"/>
-      <c r="DR3" s="40"/>
-      <c r="DS3" s="40"/>
-      <c r="DT3" s="40"/>
-      <c r="DU3" s="40"/>
-      <c r="DV3" s="40"/>
-      <c r="DW3" s="40"/>
-      <c r="DX3" s="40"/>
-      <c r="DY3" s="40"/>
-      <c r="DZ3" s="40"/>
-      <c r="EA3" s="40"/>
-      <c r="EB3" s="40"/>
-      <c r="EC3" s="40"/>
-      <c r="ED3" s="40"/>
-      <c r="EE3" s="40"/>
-      <c r="EF3" s="40"/>
-      <c r="EG3" s="40"/>
-      <c r="EH3" s="40"/>
-      <c r="EI3" s="40"/>
-      <c r="EJ3" s="40"/>
-      <c r="EK3" s="40"/>
-      <c r="EL3" s="40"/>
-      <c r="EM3" s="40"/>
-      <c r="EN3" s="40"/>
-      <c r="EO3" s="40"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="51"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="51"/>
+      <c r="S3" s="51"/>
+      <c r="T3" s="51"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="51"/>
+      <c r="W3" s="51"/>
+      <c r="X3" s="51"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="51"/>
+      <c r="AA3" s="49"/>
+      <c r="AB3" s="49"/>
+      <c r="AC3" s="39"/>
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="39"/>
+      <c r="AG3" s="39"/>
+      <c r="AH3" s="39"/>
+      <c r="AI3" s="39"/>
+      <c r="AJ3" s="39"/>
+      <c r="AK3" s="39"/>
+      <c r="AL3" s="39"/>
+      <c r="AM3" s="39"/>
+      <c r="AN3" s="39"/>
+      <c r="AO3" s="39"/>
+      <c r="AP3" s="39"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="39"/>
+      <c r="AS3" s="39"/>
+      <c r="AT3" s="39"/>
+      <c r="AU3" s="39"/>
+      <c r="AV3" s="39"/>
+      <c r="AW3" s="39"/>
+      <c r="AX3" s="39"/>
+      <c r="AY3" s="39"/>
+      <c r="AZ3" s="39"/>
+      <c r="BA3" s="39"/>
+      <c r="BB3" s="39"/>
+      <c r="BC3" s="39"/>
+      <c r="BD3" s="39"/>
+      <c r="BE3" s="39"/>
+      <c r="BF3" s="39"/>
+      <c r="BG3" s="39"/>
+      <c r="BH3" s="39"/>
+      <c r="BI3" s="39"/>
+      <c r="BJ3" s="39"/>
+      <c r="BK3" s="39"/>
+      <c r="BL3" s="39"/>
+      <c r="BM3" s="39"/>
+      <c r="BN3" s="39"/>
+      <c r="BO3" s="39"/>
+      <c r="BP3" s="39"/>
+      <c r="BQ3" s="39"/>
+      <c r="BR3" s="39"/>
+      <c r="BS3" s="39"/>
+      <c r="BT3" s="39"/>
+      <c r="BU3" s="39"/>
+      <c r="BV3" s="39"/>
+      <c r="BW3" s="39"/>
+      <c r="BX3" s="47"/>
+      <c r="BY3" s="39"/>
+      <c r="BZ3" s="39"/>
+      <c r="CA3" s="39"/>
+      <c r="CB3" s="39"/>
+      <c r="CC3" s="39"/>
+      <c r="CD3" s="39"/>
+      <c r="CE3" s="39"/>
+      <c r="CF3" s="39"/>
+      <c r="CG3" s="39"/>
+      <c r="CH3" s="39"/>
+      <c r="CI3" s="39"/>
+      <c r="CJ3" s="39"/>
+      <c r="CK3" s="39"/>
+      <c r="CL3" s="39"/>
+      <c r="CM3" s="39"/>
+      <c r="CN3" s="39"/>
+      <c r="CO3" s="39"/>
+      <c r="CP3" s="39"/>
+      <c r="CQ3" s="39"/>
+      <c r="CR3" s="39"/>
+      <c r="CS3" s="39"/>
+      <c r="CT3" s="39"/>
+      <c r="CU3" s="39"/>
+      <c r="CV3" s="39"/>
+      <c r="CW3" s="39"/>
+      <c r="CX3" s="39"/>
+      <c r="CY3" s="39"/>
+      <c r="CZ3" s="39"/>
+      <c r="DA3" s="39"/>
+      <c r="DB3" s="39"/>
+      <c r="DC3" s="39"/>
+      <c r="DD3" s="39"/>
+      <c r="DE3" s="39"/>
+      <c r="DF3" s="39"/>
+      <c r="DG3" s="39"/>
+      <c r="DH3" s="39"/>
+      <c r="DI3" s="39"/>
+      <c r="DJ3" s="39"/>
+      <c r="DK3" s="39"/>
+      <c r="DL3" s="39"/>
+      <c r="DM3" s="39"/>
+      <c r="DN3" s="39"/>
+      <c r="DO3" s="39"/>
+      <c r="DP3" s="39"/>
+      <c r="DQ3" s="39"/>
+      <c r="DR3" s="39"/>
+      <c r="DS3" s="39"/>
+      <c r="DT3" s="39"/>
+      <c r="DU3" s="39"/>
+      <c r="DV3" s="39"/>
+      <c r="DW3" s="39"/>
+      <c r="DX3" s="39"/>
+      <c r="DY3" s="39"/>
+      <c r="DZ3" s="39"/>
+      <c r="EA3" s="39"/>
+      <c r="EB3" s="39"/>
+      <c r="EC3" s="39"/>
+      <c r="ED3" s="39"/>
+      <c r="EE3" s="39"/>
+      <c r="EF3" s="39"/>
+      <c r="EG3" s="39"/>
+      <c r="EH3" s="39"/>
+      <c r="EI3" s="39"/>
+      <c r="EJ3" s="39"/>
+      <c r="EK3" s="39"/>
+      <c r="EL3" s="39"/>
+      <c r="EM3" s="39"/>
+      <c r="EN3" s="39"/>
+      <c r="EO3" s="39"/>
     </row>
-    <row r="4" spans="1:150" ht="24.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="s">
+    <row r="4" spans="1:150" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="52" t="s">
+      <c r="B4" s="41"/>
+      <c r="C4" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="53"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="40"/>
-      <c r="N4" s="40"/>
-      <c r="O4" s="40"/>
-      <c r="P4" s="40"/>
-      <c r="Q4" s="40"/>
-      <c r="R4" s="42"/>
-      <c r="S4" s="42"/>
-      <c r="T4" s="42"/>
-      <c r="U4" s="40"/>
-      <c r="V4" s="42"/>
-      <c r="W4" s="42"/>
-      <c r="X4" s="42"/>
-      <c r="Y4" s="40"/>
-      <c r="Z4" s="42"/>
-      <c r="AA4" s="47"/>
-      <c r="AB4" s="47"/>
-      <c r="AC4" s="40"/>
-      <c r="AD4" s="40"/>
-      <c r="AE4" s="40"/>
-      <c r="AF4" s="40"/>
-      <c r="AG4" s="40"/>
-      <c r="AH4" s="40"/>
-      <c r="AI4" s="40"/>
-      <c r="AJ4" s="40"/>
-      <c r="AK4" s="40"/>
-      <c r="AL4" s="40"/>
-      <c r="AM4" s="40"/>
-      <c r="AN4" s="40"/>
-      <c r="AO4" s="40"/>
-      <c r="AP4" s="40"/>
-      <c r="AQ4" s="40"/>
-      <c r="AR4" s="40"/>
-      <c r="AS4" s="40"/>
-      <c r="AT4" s="40"/>
-      <c r="AU4" s="40"/>
-      <c r="AV4" s="40"/>
-      <c r="AW4" s="40"/>
-      <c r="AX4" s="40"/>
-      <c r="AY4" s="40"/>
-      <c r="AZ4" s="40"/>
-      <c r="BA4" s="40"/>
-      <c r="BB4" s="40"/>
-      <c r="BC4" s="40"/>
-      <c r="BD4" s="40"/>
-      <c r="BE4" s="40"/>
-      <c r="BF4" s="40"/>
-      <c r="BG4" s="40"/>
-      <c r="BH4" s="40"/>
-      <c r="BI4" s="40"/>
-      <c r="BJ4" s="40"/>
-      <c r="BK4" s="40"/>
-      <c r="BL4" s="40"/>
-      <c r="BM4" s="40"/>
-      <c r="BN4" s="40"/>
-      <c r="BO4" s="40"/>
-      <c r="BP4" s="40"/>
-      <c r="BQ4" s="40"/>
-      <c r="BR4" s="40"/>
-      <c r="BS4" s="40"/>
-      <c r="BT4" s="40"/>
-      <c r="BU4" s="40"/>
-      <c r="BV4" s="40"/>
-      <c r="BW4" s="40"/>
-      <c r="BX4" s="49"/>
-      <c r="BY4" s="40"/>
-      <c r="BZ4" s="40"/>
-      <c r="CA4" s="40"/>
-      <c r="CB4" s="40"/>
-      <c r="CC4" s="40"/>
-      <c r="CD4" s="40"/>
-      <c r="CE4" s="40"/>
-      <c r="CF4" s="40"/>
-      <c r="CG4" s="40"/>
-      <c r="CH4" s="40"/>
-      <c r="CI4" s="40"/>
-      <c r="CJ4" s="40"/>
-      <c r="CK4" s="40"/>
-      <c r="CL4" s="40"/>
-      <c r="CM4" s="40"/>
-      <c r="CN4" s="40"/>
-      <c r="CO4" s="40"/>
-      <c r="CP4" s="40"/>
-      <c r="CQ4" s="40"/>
-      <c r="CR4" s="40"/>
-      <c r="CS4" s="40"/>
-      <c r="CT4" s="40"/>
-      <c r="CU4" s="40"/>
-      <c r="CV4" s="40"/>
-      <c r="CW4" s="40"/>
-      <c r="CX4" s="40"/>
-      <c r="CY4" s="40"/>
-      <c r="CZ4" s="40"/>
-      <c r="DA4" s="40"/>
-      <c r="DB4" s="40"/>
-      <c r="DC4" s="40"/>
-      <c r="DD4" s="40"/>
-      <c r="DE4" s="40"/>
-      <c r="DF4" s="40"/>
-      <c r="DG4" s="40"/>
-      <c r="DH4" s="40"/>
-      <c r="DI4" s="40"/>
-      <c r="DJ4" s="40"/>
-      <c r="DK4" s="40"/>
-      <c r="DL4" s="40"/>
-      <c r="DM4" s="40"/>
-      <c r="DN4" s="40"/>
-      <c r="DO4" s="40"/>
-      <c r="DP4" s="40"/>
-      <c r="DQ4" s="40"/>
-      <c r="DR4" s="40"/>
-      <c r="DS4" s="40"/>
-      <c r="DT4" s="40"/>
-      <c r="DU4" s="40"/>
-      <c r="DV4" s="40"/>
-      <c r="DW4" s="40"/>
-      <c r="DX4" s="40"/>
-      <c r="DY4" s="40"/>
-      <c r="DZ4" s="40"/>
-      <c r="EA4" s="40"/>
-      <c r="EB4" s="40"/>
-      <c r="EC4" s="40"/>
-      <c r="ED4" s="40"/>
-      <c r="EE4" s="40"/>
-      <c r="EF4" s="40"/>
-      <c r="EG4" s="40"/>
-      <c r="EH4" s="40"/>
-      <c r="EI4" s="40"/>
-      <c r="EJ4" s="40"/>
-      <c r="EK4" s="40"/>
-      <c r="EL4" s="40"/>
-      <c r="EM4" s="40"/>
-      <c r="EN4" s="40"/>
-      <c r="EO4" s="40"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="51"/>
+      <c r="I4" s="51"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="51"/>
+      <c r="L4" s="51"/>
+      <c r="M4" s="39"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="51"/>
+      <c r="S4" s="51"/>
+      <c r="T4" s="51"/>
+      <c r="U4" s="39"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="51"/>
+      <c r="Y4" s="39"/>
+      <c r="Z4" s="51"/>
+      <c r="AA4" s="49"/>
+      <c r="AB4" s="49"/>
+      <c r="AC4" s="39"/>
+      <c r="AD4" s="39"/>
+      <c r="AE4" s="39"/>
+      <c r="AF4" s="39"/>
+      <c r="AG4" s="39"/>
+      <c r="AH4" s="39"/>
+      <c r="AI4" s="39"/>
+      <c r="AJ4" s="39"/>
+      <c r="AK4" s="39"/>
+      <c r="AL4" s="39"/>
+      <c r="AM4" s="39"/>
+      <c r="AN4" s="39"/>
+      <c r="AO4" s="39"/>
+      <c r="AP4" s="39"/>
+      <c r="AQ4" s="39"/>
+      <c r="AR4" s="39"/>
+      <c r="AS4" s="39"/>
+      <c r="AT4" s="39"/>
+      <c r="AU4" s="39"/>
+      <c r="AV4" s="39"/>
+      <c r="AW4" s="39"/>
+      <c r="AX4" s="39"/>
+      <c r="AY4" s="39"/>
+      <c r="AZ4" s="39"/>
+      <c r="BA4" s="39"/>
+      <c r="BB4" s="39"/>
+      <c r="BC4" s="39"/>
+      <c r="BD4" s="39"/>
+      <c r="BE4" s="39"/>
+      <c r="BF4" s="39"/>
+      <c r="BG4" s="39"/>
+      <c r="BH4" s="39"/>
+      <c r="BI4" s="39"/>
+      <c r="BJ4" s="39"/>
+      <c r="BK4" s="39"/>
+      <c r="BL4" s="39"/>
+      <c r="BM4" s="39"/>
+      <c r="BN4" s="39"/>
+      <c r="BO4" s="39"/>
+      <c r="BP4" s="39"/>
+      <c r="BQ4" s="39"/>
+      <c r="BR4" s="39"/>
+      <c r="BS4" s="39"/>
+      <c r="BT4" s="39"/>
+      <c r="BU4" s="39"/>
+      <c r="BV4" s="39"/>
+      <c r="BW4" s="39"/>
+      <c r="BX4" s="47"/>
+      <c r="BY4" s="39"/>
+      <c r="BZ4" s="39"/>
+      <c r="CA4" s="39"/>
+      <c r="CB4" s="39"/>
+      <c r="CC4" s="39"/>
+      <c r="CD4" s="39"/>
+      <c r="CE4" s="39"/>
+      <c r="CF4" s="39"/>
+      <c r="CG4" s="39"/>
+      <c r="CH4" s="39"/>
+      <c r="CI4" s="39"/>
+      <c r="CJ4" s="39"/>
+      <c r="CK4" s="39"/>
+      <c r="CL4" s="39"/>
+      <c r="CM4" s="39"/>
+      <c r="CN4" s="39"/>
+      <c r="CO4" s="39"/>
+      <c r="CP4" s="39"/>
+      <c r="CQ4" s="39"/>
+      <c r="CR4" s="39"/>
+      <c r="CS4" s="39"/>
+      <c r="CT4" s="39"/>
+      <c r="CU4" s="39"/>
+      <c r="CV4" s="39"/>
+      <c r="CW4" s="39"/>
+      <c r="CX4" s="39"/>
+      <c r="CY4" s="39"/>
+      <c r="CZ4" s="39"/>
+      <c r="DA4" s="39"/>
+      <c r="DB4" s="39"/>
+      <c r="DC4" s="39"/>
+      <c r="DD4" s="39"/>
+      <c r="DE4" s="39"/>
+      <c r="DF4" s="39"/>
+      <c r="DG4" s="39"/>
+      <c r="DH4" s="39"/>
+      <c r="DI4" s="39"/>
+      <c r="DJ4" s="39"/>
+      <c r="DK4" s="39"/>
+      <c r="DL4" s="39"/>
+      <c r="DM4" s="39"/>
+      <c r="DN4" s="39"/>
+      <c r="DO4" s="39"/>
+      <c r="DP4" s="39"/>
+      <c r="DQ4" s="39"/>
+      <c r="DR4" s="39"/>
+      <c r="DS4" s="39"/>
+      <c r="DT4" s="39"/>
+      <c r="DU4" s="39"/>
+      <c r="DV4" s="39"/>
+      <c r="DW4" s="39"/>
+      <c r="DX4" s="39"/>
+      <c r="DY4" s="39"/>
+      <c r="DZ4" s="39"/>
+      <c r="EA4" s="39"/>
+      <c r="EB4" s="39"/>
+      <c r="EC4" s="39"/>
+      <c r="ED4" s="39"/>
+      <c r="EE4" s="39"/>
+      <c r="EF4" s="39"/>
+      <c r="EG4" s="39"/>
+      <c r="EH4" s="39"/>
+      <c r="EI4" s="39"/>
+      <c r="EJ4" s="39"/>
+      <c r="EK4" s="39"/>
+      <c r="EL4" s="39"/>
+      <c r="EM4" s="39"/>
+      <c r="EN4" s="39"/>
+      <c r="EO4" s="39"/>
     </row>
-    <row r="5" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="54" t="s">
+    <row r="5" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="55">
+      <c r="B5" s="43"/>
+      <c r="C5" s="44">
         <v>110</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="42"/>
-      <c r="L5" s="42"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="40"/>
-      <c r="O5" s="40"/>
-      <c r="P5" s="40"/>
-      <c r="Q5" s="40"/>
-      <c r="R5" s="42"/>
-      <c r="S5" s="42"/>
-      <c r="T5" s="42"/>
-      <c r="U5" s="40"/>
-      <c r="V5" s="42"/>
-      <c r="W5" s="42"/>
-      <c r="X5" s="42"/>
-      <c r="Y5" s="40"/>
-      <c r="Z5" s="42"/>
-      <c r="AA5" s="47"/>
-      <c r="AB5" s="47"/>
-      <c r="AC5" s="40"/>
-      <c r="AD5" s="40"/>
-      <c r="AE5" s="40"/>
-      <c r="AF5" s="40"/>
-      <c r="AG5" s="40"/>
-      <c r="AH5" s="40"/>
-      <c r="AI5" s="40"/>
-      <c r="AJ5" s="40"/>
-      <c r="AK5" s="40"/>
-      <c r="AL5" s="40"/>
-      <c r="AM5" s="40"/>
-      <c r="AN5" s="40"/>
-      <c r="AO5" s="40"/>
-      <c r="AP5" s="40"/>
-      <c r="AQ5" s="40"/>
-      <c r="AR5" s="40"/>
-      <c r="AS5" s="40"/>
-      <c r="AT5" s="40"/>
-      <c r="AU5" s="40"/>
-      <c r="AV5" s="40"/>
-      <c r="AW5" s="40"/>
-      <c r="AX5" s="40"/>
-      <c r="AY5" s="40"/>
-      <c r="AZ5" s="40"/>
-      <c r="BA5" s="40"/>
-      <c r="BB5" s="40"/>
-      <c r="BC5" s="40"/>
-      <c r="BD5" s="40"/>
-      <c r="BE5" s="40"/>
-      <c r="BF5" s="40"/>
-      <c r="BG5" s="40"/>
-      <c r="BH5" s="40"/>
-      <c r="BI5" s="40"/>
-      <c r="BJ5" s="40"/>
-      <c r="BK5" s="40"/>
-      <c r="BL5" s="40"/>
-      <c r="BM5" s="40"/>
-      <c r="BN5" s="40"/>
-      <c r="BO5" s="40"/>
-      <c r="BP5" s="40"/>
-      <c r="BQ5" s="40"/>
-      <c r="BR5" s="40"/>
-      <c r="BS5" s="40"/>
-      <c r="BT5" s="40"/>
-      <c r="BU5" s="40"/>
-      <c r="BV5" s="40"/>
-      <c r="BW5" s="40"/>
-      <c r="BX5" s="49"/>
-      <c r="BY5" s="40"/>
-      <c r="BZ5" s="40"/>
-      <c r="CA5" s="40"/>
-      <c r="CB5" s="40"/>
-      <c r="CC5" s="40"/>
-      <c r="CD5" s="40"/>
-      <c r="CE5" s="40"/>
-      <c r="CF5" s="40"/>
-      <c r="CG5" s="40"/>
-      <c r="CH5" s="40"/>
-      <c r="CI5" s="40"/>
-      <c r="CJ5" s="40"/>
-      <c r="CK5" s="40"/>
-      <c r="CL5" s="40"/>
-      <c r="CM5" s="40"/>
-      <c r="CN5" s="40"/>
-      <c r="CO5" s="40"/>
-      <c r="CP5" s="40"/>
-      <c r="CQ5" s="40"/>
-      <c r="CR5" s="40"/>
-      <c r="CS5" s="40"/>
-      <c r="CT5" s="40"/>
-      <c r="CU5" s="40"/>
-      <c r="CV5" s="40"/>
-      <c r="CW5" s="40"/>
-      <c r="CX5" s="40"/>
-      <c r="CY5" s="40"/>
-      <c r="CZ5" s="40"/>
-      <c r="DA5" s="40"/>
-      <c r="DB5" s="40"/>
-      <c r="DC5" s="40"/>
-      <c r="DD5" s="40"/>
-      <c r="DE5" s="40"/>
-      <c r="DF5" s="40"/>
-      <c r="DG5" s="40"/>
-      <c r="DH5" s="40"/>
-      <c r="DI5" s="40"/>
-      <c r="DJ5" s="40"/>
-      <c r="DK5" s="40"/>
-      <c r="DL5" s="40"/>
-      <c r="DM5" s="40"/>
-      <c r="DN5" s="40"/>
-      <c r="DO5" s="40"/>
-      <c r="DP5" s="40"/>
-      <c r="DQ5" s="40"/>
-      <c r="DR5" s="40"/>
-      <c r="DS5" s="40"/>
-      <c r="DT5" s="40"/>
-      <c r="DU5" s="40"/>
-      <c r="DV5" s="40"/>
-      <c r="DW5" s="40"/>
-      <c r="DX5" s="40"/>
-      <c r="DY5" s="40"/>
-      <c r="DZ5" s="40"/>
-      <c r="EA5" s="40"/>
-      <c r="EB5" s="40"/>
-      <c r="EC5" s="40"/>
-      <c r="ED5" s="40"/>
-      <c r="EE5" s="40"/>
-      <c r="EF5" s="40"/>
-      <c r="EG5" s="40"/>
-      <c r="EH5" s="40"/>
-      <c r="EI5" s="40"/>
-      <c r="EJ5" s="40"/>
-      <c r="EK5" s="40"/>
-      <c r="EL5" s="40"/>
-      <c r="EM5" s="40"/>
-      <c r="EN5" s="40"/>
-      <c r="EO5" s="40"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="67"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="51"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="39"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="39"/>
+      <c r="P5" s="39"/>
+      <c r="Q5" s="39"/>
+      <c r="R5" s="51"/>
+      <c r="S5" s="51"/>
+      <c r="T5" s="51"/>
+      <c r="U5" s="39"/>
+      <c r="V5" s="51"/>
+      <c r="W5" s="51"/>
+      <c r="X5" s="51"/>
+      <c r="Y5" s="39"/>
+      <c r="Z5" s="51"/>
+      <c r="AA5" s="49"/>
+      <c r="AB5" s="49"/>
+      <c r="AC5" s="39"/>
+      <c r="AD5" s="39"/>
+      <c r="AE5" s="39"/>
+      <c r="AF5" s="39"/>
+      <c r="AG5" s="39"/>
+      <c r="AH5" s="39"/>
+      <c r="AI5" s="39"/>
+      <c r="AJ5" s="39"/>
+      <c r="AK5" s="39"/>
+      <c r="AL5" s="39"/>
+      <c r="AM5" s="39"/>
+      <c r="AN5" s="39"/>
+      <c r="AO5" s="39"/>
+      <c r="AP5" s="39"/>
+      <c r="AQ5" s="39"/>
+      <c r="AR5" s="39"/>
+      <c r="AS5" s="39"/>
+      <c r="AT5" s="39"/>
+      <c r="AU5" s="39"/>
+      <c r="AV5" s="39"/>
+      <c r="AW5" s="39"/>
+      <c r="AX5" s="39"/>
+      <c r="AY5" s="39"/>
+      <c r="AZ5" s="39"/>
+      <c r="BA5" s="39"/>
+      <c r="BB5" s="39"/>
+      <c r="BC5" s="39"/>
+      <c r="BD5" s="39"/>
+      <c r="BE5" s="39"/>
+      <c r="BF5" s="39"/>
+      <c r="BG5" s="39"/>
+      <c r="BH5" s="39"/>
+      <c r="BI5" s="39"/>
+      <c r="BJ5" s="39"/>
+      <c r="BK5" s="39"/>
+      <c r="BL5" s="39"/>
+      <c r="BM5" s="39"/>
+      <c r="BN5" s="39"/>
+      <c r="BO5" s="39"/>
+      <c r="BP5" s="39"/>
+      <c r="BQ5" s="39"/>
+      <c r="BR5" s="39"/>
+      <c r="BS5" s="39"/>
+      <c r="BT5" s="39"/>
+      <c r="BU5" s="39"/>
+      <c r="BV5" s="39"/>
+      <c r="BW5" s="39"/>
+      <c r="BX5" s="47"/>
+      <c r="BY5" s="39"/>
+      <c r="BZ5" s="39"/>
+      <c r="CA5" s="39"/>
+      <c r="CB5" s="39"/>
+      <c r="CC5" s="39"/>
+      <c r="CD5" s="39"/>
+      <c r="CE5" s="39"/>
+      <c r="CF5" s="39"/>
+      <c r="CG5" s="39"/>
+      <c r="CH5" s="39"/>
+      <c r="CI5" s="39"/>
+      <c r="CJ5" s="39"/>
+      <c r="CK5" s="39"/>
+      <c r="CL5" s="39"/>
+      <c r="CM5" s="39"/>
+      <c r="CN5" s="39"/>
+      <c r="CO5" s="39"/>
+      <c r="CP5" s="39"/>
+      <c r="CQ5" s="39"/>
+      <c r="CR5" s="39"/>
+      <c r="CS5" s="39"/>
+      <c r="CT5" s="39"/>
+      <c r="CU5" s="39"/>
+      <c r="CV5" s="39"/>
+      <c r="CW5" s="39"/>
+      <c r="CX5" s="39"/>
+      <c r="CY5" s="39"/>
+      <c r="CZ5" s="39"/>
+      <c r="DA5" s="39"/>
+      <c r="DB5" s="39"/>
+      <c r="DC5" s="39"/>
+      <c r="DD5" s="39"/>
+      <c r="DE5" s="39"/>
+      <c r="DF5" s="39"/>
+      <c r="DG5" s="39"/>
+      <c r="DH5" s="39"/>
+      <c r="DI5" s="39"/>
+      <c r="DJ5" s="39"/>
+      <c r="DK5" s="39"/>
+      <c r="DL5" s="39"/>
+      <c r="DM5" s="39"/>
+      <c r="DN5" s="39"/>
+      <c r="DO5" s="39"/>
+      <c r="DP5" s="39"/>
+      <c r="DQ5" s="39"/>
+      <c r="DR5" s="39"/>
+      <c r="DS5" s="39"/>
+      <c r="DT5" s="39"/>
+      <c r="DU5" s="39"/>
+      <c r="DV5" s="39"/>
+      <c r="DW5" s="39"/>
+      <c r="DX5" s="39"/>
+      <c r="DY5" s="39"/>
+      <c r="DZ5" s="39"/>
+      <c r="EA5" s="39"/>
+      <c r="EB5" s="39"/>
+      <c r="EC5" s="39"/>
+      <c r="ED5" s="39"/>
+      <c r="EE5" s="39"/>
+      <c r="EF5" s="39"/>
+      <c r="EG5" s="39"/>
+      <c r="EH5" s="39"/>
+      <c r="EI5" s="39"/>
+      <c r="EJ5" s="39"/>
+      <c r="EK5" s="39"/>
+      <c r="EL5" s="39"/>
+      <c r="EM5" s="39"/>
+      <c r="EN5" s="39"/>
+      <c r="EO5" s="39"/>
     </row>
-    <row r="6" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54" t="s">
+    <row r="6" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="55">
+      <c r="B6" s="43"/>
+      <c r="C6" s="44">
         <v>10</v>
       </c>
-      <c r="D6" s="56"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="42"/>
-      <c r="M6" s="40"/>
-      <c r="N6" s="40"/>
-      <c r="O6" s="40"/>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="40"/>
-      <c r="R6" s="42"/>
-      <c r="S6" s="42"/>
-      <c r="T6" s="42"/>
-      <c r="U6" s="40"/>
-      <c r="V6" s="42"/>
-      <c r="W6" s="42"/>
-      <c r="X6" s="42"/>
-      <c r="Y6" s="40"/>
-      <c r="Z6" s="42"/>
-      <c r="AA6" s="47"/>
-      <c r="AB6" s="47"/>
-      <c r="AC6" s="40"/>
-      <c r="AD6" s="40"/>
-      <c r="AE6" s="40"/>
-      <c r="AF6" s="40"/>
-      <c r="AG6" s="40"/>
-      <c r="AH6" s="40"/>
-      <c r="AI6" s="40"/>
-      <c r="AJ6" s="40"/>
-      <c r="AK6" s="40"/>
-      <c r="AL6" s="40"/>
-      <c r="AM6" s="40"/>
-      <c r="AN6" s="40"/>
-      <c r="AO6" s="40"/>
-      <c r="AP6" s="40"/>
-      <c r="AQ6" s="40"/>
-      <c r="AR6" s="40"/>
-      <c r="AS6" s="40"/>
-      <c r="AT6" s="40"/>
-      <c r="AU6" s="40"/>
-      <c r="AV6" s="40"/>
-      <c r="AW6" s="40"/>
-      <c r="AX6" s="40"/>
-      <c r="AY6" s="40"/>
-      <c r="AZ6" s="40"/>
-      <c r="BA6" s="40"/>
-      <c r="BB6" s="40"/>
-      <c r="BC6" s="40"/>
-      <c r="BD6" s="40"/>
-      <c r="BE6" s="40"/>
-      <c r="BF6" s="40"/>
-      <c r="BG6" s="40"/>
-      <c r="BH6" s="40"/>
-      <c r="BI6" s="40"/>
-      <c r="BJ6" s="40"/>
-      <c r="BK6" s="40"/>
-      <c r="BL6" s="40"/>
-      <c r="BM6" s="40"/>
-      <c r="BN6" s="40"/>
-      <c r="BO6" s="40"/>
-      <c r="BP6" s="40"/>
-      <c r="BQ6" s="40"/>
-      <c r="BR6" s="40"/>
-      <c r="BS6" s="40"/>
-      <c r="BT6" s="40"/>
-      <c r="BU6" s="40"/>
-      <c r="BV6" s="40"/>
-      <c r="BW6" s="40"/>
-      <c r="BX6" s="49"/>
-      <c r="BY6" s="40"/>
-      <c r="BZ6" s="40"/>
-      <c r="CA6" s="40"/>
-      <c r="CB6" s="40"/>
-      <c r="CC6" s="40"/>
-      <c r="CD6" s="40"/>
-      <c r="CE6" s="40"/>
-      <c r="CF6" s="40"/>
-      <c r="CG6" s="40"/>
-      <c r="CH6" s="40"/>
-      <c r="CI6" s="40"/>
-      <c r="CJ6" s="40"/>
-      <c r="CK6" s="40"/>
-      <c r="CL6" s="40"/>
-      <c r="CM6" s="40"/>
-      <c r="CN6" s="40"/>
-      <c r="CO6" s="40"/>
-      <c r="CP6" s="40"/>
-      <c r="CQ6" s="40"/>
-      <c r="CR6" s="40"/>
-      <c r="CS6" s="40"/>
-      <c r="CT6" s="40"/>
-      <c r="CU6" s="40"/>
-      <c r="CV6" s="40"/>
-      <c r="CW6" s="40"/>
-      <c r="CX6" s="40"/>
-      <c r="CY6" s="40"/>
-      <c r="CZ6" s="40"/>
-      <c r="DA6" s="40"/>
-      <c r="DB6" s="40"/>
-      <c r="DC6" s="40"/>
-      <c r="DD6" s="40"/>
-      <c r="DE6" s="40"/>
-      <c r="DF6" s="40"/>
-      <c r="DG6" s="40"/>
-      <c r="DH6" s="40"/>
-      <c r="DI6" s="40"/>
-      <c r="DJ6" s="40"/>
-      <c r="DK6" s="40"/>
-      <c r="DL6" s="40"/>
-      <c r="DM6" s="40"/>
-      <c r="DN6" s="40"/>
-      <c r="DO6" s="40"/>
-      <c r="DP6" s="40"/>
-      <c r="DQ6" s="40"/>
-      <c r="DR6" s="40"/>
-      <c r="DS6" s="40"/>
-      <c r="DT6" s="40"/>
-      <c r="DU6" s="40"/>
-      <c r="DV6" s="40"/>
-      <c r="DW6" s="40"/>
-      <c r="DX6" s="40"/>
-      <c r="DY6" s="40"/>
-      <c r="DZ6" s="40"/>
-      <c r="EA6" s="40"/>
-      <c r="EB6" s="40"/>
-      <c r="EC6" s="40"/>
-      <c r="ED6" s="40"/>
-      <c r="EE6" s="40"/>
-      <c r="EF6" s="40"/>
-      <c r="EG6" s="40"/>
-      <c r="EH6" s="40"/>
-      <c r="EI6" s="40"/>
-      <c r="EJ6" s="40"/>
-      <c r="EK6" s="40"/>
-      <c r="EL6" s="40"/>
-      <c r="EM6" s="40"/>
-      <c r="EN6" s="40"/>
-      <c r="EO6" s="40"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="51"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="39"/>
+      <c r="P6" s="39"/>
+      <c r="Q6" s="39"/>
+      <c r="R6" s="51"/>
+      <c r="S6" s="51"/>
+      <c r="T6" s="51"/>
+      <c r="U6" s="39"/>
+      <c r="V6" s="51"/>
+      <c r="W6" s="51"/>
+      <c r="X6" s="51"/>
+      <c r="Y6" s="39"/>
+      <c r="Z6" s="51"/>
+      <c r="AA6" s="49"/>
+      <c r="AB6" s="49"/>
+      <c r="AC6" s="39"/>
+      <c r="AD6" s="39"/>
+      <c r="AE6" s="39"/>
+      <c r="AF6" s="39"/>
+      <c r="AG6" s="39"/>
+      <c r="AH6" s="39"/>
+      <c r="AI6" s="39"/>
+      <c r="AJ6" s="39"/>
+      <c r="AK6" s="39"/>
+      <c r="AL6" s="39"/>
+      <c r="AM6" s="39"/>
+      <c r="AN6" s="39"/>
+      <c r="AO6" s="39"/>
+      <c r="AP6" s="39"/>
+      <c r="AQ6" s="39"/>
+      <c r="AR6" s="39"/>
+      <c r="AS6" s="39"/>
+      <c r="AT6" s="39"/>
+      <c r="AU6" s="39"/>
+      <c r="AV6" s="39"/>
+      <c r="AW6" s="39"/>
+      <c r="AX6" s="39"/>
+      <c r="AY6" s="39"/>
+      <c r="AZ6" s="39"/>
+      <c r="BA6" s="39"/>
+      <c r="BB6" s="39"/>
+      <c r="BC6" s="39"/>
+      <c r="BD6" s="39"/>
+      <c r="BE6" s="39"/>
+      <c r="BF6" s="39"/>
+      <c r="BG6" s="39"/>
+      <c r="BH6" s="39"/>
+      <c r="BI6" s="39"/>
+      <c r="BJ6" s="39"/>
+      <c r="BK6" s="39"/>
+      <c r="BL6" s="39"/>
+      <c r="BM6" s="39"/>
+      <c r="BN6" s="39"/>
+      <c r="BO6" s="39"/>
+      <c r="BP6" s="39"/>
+      <c r="BQ6" s="39"/>
+      <c r="BR6" s="39"/>
+      <c r="BS6" s="39"/>
+      <c r="BT6" s="39"/>
+      <c r="BU6" s="39"/>
+      <c r="BV6" s="39"/>
+      <c r="BW6" s="39"/>
+      <c r="BX6" s="47"/>
+      <c r="BY6" s="39"/>
+      <c r="BZ6" s="39"/>
+      <c r="CA6" s="39"/>
+      <c r="CB6" s="39"/>
+      <c r="CC6" s="39"/>
+      <c r="CD6" s="39"/>
+      <c r="CE6" s="39"/>
+      <c r="CF6" s="39"/>
+      <c r="CG6" s="39"/>
+      <c r="CH6" s="39"/>
+      <c r="CI6" s="39"/>
+      <c r="CJ6" s="39"/>
+      <c r="CK6" s="39"/>
+      <c r="CL6" s="39"/>
+      <c r="CM6" s="39"/>
+      <c r="CN6" s="39"/>
+      <c r="CO6" s="39"/>
+      <c r="CP6" s="39"/>
+      <c r="CQ6" s="39"/>
+      <c r="CR6" s="39"/>
+      <c r="CS6" s="39"/>
+      <c r="CT6" s="39"/>
+      <c r="CU6" s="39"/>
+      <c r="CV6" s="39"/>
+      <c r="CW6" s="39"/>
+      <c r="CX6" s="39"/>
+      <c r="CY6" s="39"/>
+      <c r="CZ6" s="39"/>
+      <c r="DA6" s="39"/>
+      <c r="DB6" s="39"/>
+      <c r="DC6" s="39"/>
+      <c r="DD6" s="39"/>
+      <c r="DE6" s="39"/>
+      <c r="DF6" s="39"/>
+      <c r="DG6" s="39"/>
+      <c r="DH6" s="39"/>
+      <c r="DI6" s="39"/>
+      <c r="DJ6" s="39"/>
+      <c r="DK6" s="39"/>
+      <c r="DL6" s="39"/>
+      <c r="DM6" s="39"/>
+      <c r="DN6" s="39"/>
+      <c r="DO6" s="39"/>
+      <c r="DP6" s="39"/>
+      <c r="DQ6" s="39"/>
+      <c r="DR6" s="39"/>
+      <c r="DS6" s="39"/>
+      <c r="DT6" s="39"/>
+      <c r="DU6" s="39"/>
+      <c r="DV6" s="39"/>
+      <c r="DW6" s="39"/>
+      <c r="DX6" s="39"/>
+      <c r="DY6" s="39"/>
+      <c r="DZ6" s="39"/>
+      <c r="EA6" s="39"/>
+      <c r="EB6" s="39"/>
+      <c r="EC6" s="39"/>
+      <c r="ED6" s="39"/>
+      <c r="EE6" s="39"/>
+      <c r="EF6" s="39"/>
+      <c r="EG6" s="39"/>
+      <c r="EH6" s="39"/>
+      <c r="EI6" s="39"/>
+      <c r="EJ6" s="39"/>
+      <c r="EK6" s="39"/>
+      <c r="EL6" s="39"/>
+      <c r="EM6" s="39"/>
+      <c r="EN6" s="39"/>
+      <c r="EO6" s="39"/>
     </row>
-    <row r="7" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="57" t="s">
+    <row r="7" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="57"/>
-      <c r="C7" s="55">
+      <c r="B7" s="46"/>
+      <c r="C7" s="44">
         <v>30</v>
       </c>
-      <c r="D7" s="56"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="41"/>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="43"/>
-      <c r="S7" s="43"/>
-      <c r="T7" s="43"/>
-      <c r="U7" s="41"/>
-      <c r="V7" s="43"/>
-      <c r="W7" s="43"/>
-      <c r="X7" s="43"/>
-      <c r="Y7" s="41"/>
-      <c r="Z7" s="43"/>
-      <c r="AA7" s="48"/>
-      <c r="AB7" s="48"/>
-      <c r="AC7" s="41"/>
-      <c r="AD7" s="41"/>
-      <c r="AE7" s="41"/>
-      <c r="AF7" s="41"/>
-      <c r="AG7" s="41"/>
-      <c r="AH7" s="41"/>
-      <c r="AI7" s="41"/>
-      <c r="AJ7" s="41"/>
-      <c r="AK7" s="41"/>
-      <c r="AL7" s="41"/>
-      <c r="AM7" s="41"/>
-      <c r="AN7" s="41"/>
-      <c r="AO7" s="41"/>
-      <c r="AP7" s="41"/>
-      <c r="AQ7" s="41"/>
-      <c r="AR7" s="41"/>
-      <c r="AS7" s="41"/>
-      <c r="AT7" s="41"/>
-      <c r="AU7" s="41"/>
-      <c r="AV7" s="41"/>
-      <c r="AW7" s="41"/>
-      <c r="AX7" s="41"/>
-      <c r="AY7" s="41"/>
-      <c r="AZ7" s="41"/>
-      <c r="BA7" s="41"/>
-      <c r="BB7" s="41"/>
-      <c r="BC7" s="41"/>
-      <c r="BD7" s="41"/>
-      <c r="BE7" s="41"/>
-      <c r="BF7" s="41"/>
-      <c r="BG7" s="41"/>
-      <c r="BH7" s="41"/>
-      <c r="BI7" s="41"/>
-      <c r="BJ7" s="41"/>
-      <c r="BK7" s="41"/>
-      <c r="BL7" s="41"/>
-      <c r="BM7" s="41"/>
-      <c r="BN7" s="41"/>
-      <c r="BO7" s="41"/>
-      <c r="BP7" s="41"/>
-      <c r="BQ7" s="41"/>
-      <c r="BR7" s="41"/>
-      <c r="BS7" s="41"/>
-      <c r="BT7" s="41"/>
-      <c r="BU7" s="41"/>
-      <c r="BV7" s="41"/>
-      <c r="BW7" s="41"/>
-      <c r="BX7" s="50"/>
-      <c r="BY7" s="41"/>
-      <c r="BZ7" s="41"/>
-      <c r="CA7" s="41"/>
-      <c r="CB7" s="41"/>
-      <c r="CC7" s="41"/>
-      <c r="CD7" s="41"/>
-      <c r="CE7" s="41"/>
-      <c r="CF7" s="41"/>
-      <c r="CG7" s="41"/>
-      <c r="CH7" s="41"/>
-      <c r="CI7" s="41"/>
-      <c r="CJ7" s="41"/>
-      <c r="CK7" s="41"/>
-      <c r="CL7" s="41"/>
-      <c r="CM7" s="41"/>
-      <c r="CN7" s="41"/>
-      <c r="CO7" s="41"/>
-      <c r="CP7" s="41"/>
-      <c r="CQ7" s="41"/>
-      <c r="CR7" s="41"/>
-      <c r="CS7" s="41"/>
-      <c r="CT7" s="41"/>
-      <c r="CU7" s="41"/>
-      <c r="CV7" s="41"/>
-      <c r="CW7" s="41"/>
-      <c r="CX7" s="41"/>
-      <c r="CY7" s="41"/>
-      <c r="CZ7" s="41"/>
-      <c r="DA7" s="41"/>
-      <c r="DB7" s="41"/>
-      <c r="DC7" s="41"/>
-      <c r="DD7" s="41"/>
-      <c r="DE7" s="41"/>
-      <c r="DF7" s="41"/>
-      <c r="DG7" s="41"/>
-      <c r="DH7" s="41"/>
-      <c r="DI7" s="41"/>
-      <c r="DJ7" s="41"/>
-      <c r="DK7" s="41"/>
-      <c r="DL7" s="41"/>
-      <c r="DM7" s="41"/>
-      <c r="DN7" s="41"/>
-      <c r="DO7" s="41"/>
-      <c r="DP7" s="41"/>
-      <c r="DQ7" s="41"/>
-      <c r="DR7" s="41"/>
-      <c r="DS7" s="41"/>
-      <c r="DT7" s="41"/>
-      <c r="DU7" s="41"/>
-      <c r="DV7" s="41"/>
-      <c r="DW7" s="41"/>
-      <c r="DX7" s="41"/>
-      <c r="DY7" s="41"/>
-      <c r="DZ7" s="41"/>
-      <c r="EA7" s="41"/>
-      <c r="EB7" s="41"/>
-      <c r="EC7" s="41"/>
-      <c r="ED7" s="41"/>
-      <c r="EE7" s="41"/>
-      <c r="EF7" s="41"/>
-      <c r="EG7" s="41"/>
-      <c r="EH7" s="41"/>
-      <c r="EI7" s="41"/>
-      <c r="EJ7" s="41"/>
-      <c r="EK7" s="41"/>
-      <c r="EL7" s="41"/>
-      <c r="EM7" s="41"/>
-      <c r="EN7" s="41"/>
-      <c r="EO7" s="41"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="52"/>
+      <c r="M7" s="40"/>
+      <c r="N7" s="40"/>
+      <c r="O7" s="40"/>
+      <c r="P7" s="40"/>
+      <c r="Q7" s="40"/>
+      <c r="R7" s="52"/>
+      <c r="S7" s="52"/>
+      <c r="T7" s="52"/>
+      <c r="U7" s="40"/>
+      <c r="V7" s="52"/>
+      <c r="W7" s="52"/>
+      <c r="X7" s="52"/>
+      <c r="Y7" s="40"/>
+      <c r="Z7" s="52"/>
+      <c r="AA7" s="50"/>
+      <c r="AB7" s="50"/>
+      <c r="AC7" s="40"/>
+      <c r="AD7" s="40"/>
+      <c r="AE7" s="40"/>
+      <c r="AF7" s="40"/>
+      <c r="AG7" s="40"/>
+      <c r="AH7" s="40"/>
+      <c r="AI7" s="40"/>
+      <c r="AJ7" s="40"/>
+      <c r="AK7" s="40"/>
+      <c r="AL7" s="40"/>
+      <c r="AM7" s="40"/>
+      <c r="AN7" s="40"/>
+      <c r="AO7" s="40"/>
+      <c r="AP7" s="40"/>
+      <c r="AQ7" s="40"/>
+      <c r="AR7" s="40"/>
+      <c r="AS7" s="40"/>
+      <c r="AT7" s="40"/>
+      <c r="AU7" s="40"/>
+      <c r="AV7" s="40"/>
+      <c r="AW7" s="40"/>
+      <c r="AX7" s="40"/>
+      <c r="AY7" s="40"/>
+      <c r="AZ7" s="40"/>
+      <c r="BA7" s="40"/>
+      <c r="BB7" s="40"/>
+      <c r="BC7" s="40"/>
+      <c r="BD7" s="40"/>
+      <c r="BE7" s="40"/>
+      <c r="BF7" s="40"/>
+      <c r="BG7" s="40"/>
+      <c r="BH7" s="40"/>
+      <c r="BI7" s="40"/>
+      <c r="BJ7" s="40"/>
+      <c r="BK7" s="40"/>
+      <c r="BL7" s="40"/>
+      <c r="BM7" s="40"/>
+      <c r="BN7" s="40"/>
+      <c r="BO7" s="40"/>
+      <c r="BP7" s="40"/>
+      <c r="BQ7" s="40"/>
+      <c r="BR7" s="40"/>
+      <c r="BS7" s="40"/>
+      <c r="BT7" s="40"/>
+      <c r="BU7" s="40"/>
+      <c r="BV7" s="40"/>
+      <c r="BW7" s="40"/>
+      <c r="BX7" s="48"/>
+      <c r="BY7" s="40"/>
+      <c r="BZ7" s="40"/>
+      <c r="CA7" s="40"/>
+      <c r="CB7" s="40"/>
+      <c r="CC7" s="40"/>
+      <c r="CD7" s="40"/>
+      <c r="CE7" s="40"/>
+      <c r="CF7" s="40"/>
+      <c r="CG7" s="40"/>
+      <c r="CH7" s="40"/>
+      <c r="CI7" s="40"/>
+      <c r="CJ7" s="40"/>
+      <c r="CK7" s="40"/>
+      <c r="CL7" s="40"/>
+      <c r="CM7" s="40"/>
+      <c r="CN7" s="40"/>
+      <c r="CO7" s="40"/>
+      <c r="CP7" s="40"/>
+      <c r="CQ7" s="40"/>
+      <c r="CR7" s="40"/>
+      <c r="CS7" s="40"/>
+      <c r="CT7" s="40"/>
+      <c r="CU7" s="40"/>
+      <c r="CV7" s="40"/>
+      <c r="CW7" s="40"/>
+      <c r="CX7" s="40"/>
+      <c r="CY7" s="40"/>
+      <c r="CZ7" s="40"/>
+      <c r="DA7" s="40"/>
+      <c r="DB7" s="40"/>
+      <c r="DC7" s="40"/>
+      <c r="DD7" s="40"/>
+      <c r="DE7" s="40"/>
+      <c r="DF7" s="40"/>
+      <c r="DG7" s="40"/>
+      <c r="DH7" s="40"/>
+      <c r="DI7" s="40"/>
+      <c r="DJ7" s="40"/>
+      <c r="DK7" s="40"/>
+      <c r="DL7" s="40"/>
+      <c r="DM7" s="40"/>
+      <c r="DN7" s="40"/>
+      <c r="DO7" s="40"/>
+      <c r="DP7" s="40"/>
+      <c r="DQ7" s="40"/>
+      <c r="DR7" s="40"/>
+      <c r="DS7" s="40"/>
+      <c r="DT7" s="40"/>
+      <c r="DU7" s="40"/>
+      <c r="DV7" s="40"/>
+      <c r="DW7" s="40"/>
+      <c r="DX7" s="40"/>
+      <c r="DY7" s="40"/>
+      <c r="DZ7" s="40"/>
+      <c r="EA7" s="40"/>
+      <c r="EB7" s="40"/>
+      <c r="EC7" s="40"/>
+      <c r="ED7" s="40"/>
+      <c r="EE7" s="40"/>
+      <c r="EF7" s="40"/>
+      <c r="EG7" s="40"/>
+      <c r="EH7" s="40"/>
+      <c r="EI7" s="40"/>
+      <c r="EJ7" s="40"/>
+      <c r="EK7" s="40"/>
+      <c r="EL7" s="40"/>
+      <c r="EM7" s="40"/>
+      <c r="EN7" s="40"/>
+      <c r="EO7" s="40"/>
     </row>
-    <row r="8" spans="1:150" ht="23.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="58" t="s">
+    <row r="8" spans="1:150" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="59">
+      <c r="B8" s="33"/>
+      <c r="C8" s="34">
         <v>150</v>
       </c>
-      <c r="D8" s="53"/>
+      <c r="D8" s="35"/>
       <c r="E8" s="6"/>
-      <c r="F8" s="60">
+      <c r="F8" s="27">
         <v>1</v>
       </c>
-      <c r="G8" s="60">
+      <c r="G8" s="27">
         <v>2</v>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="27">
         <v>3</v>
       </c>
-      <c r="I8" s="60">
+      <c r="I8" s="27">
         <v>4</v>
       </c>
-      <c r="J8" s="60">
+      <c r="J8" s="27">
         <v>5</v>
       </c>
-      <c r="K8" s="60">
+      <c r="K8" s="27">
         <v>6</v>
       </c>
-      <c r="L8" s="60">
+      <c r="L8" s="27">
         <v>7</v>
       </c>
-      <c r="M8" s="60">
+      <c r="M8" s="27">
         <v>8</v>
       </c>
-      <c r="N8" s="60">
+      <c r="N8" s="27">
         <v>9</v>
       </c>
-      <c r="O8" s="60">
+      <c r="O8" s="27">
         <v>10</v>
       </c>
-      <c r="P8" s="60">
+      <c r="P8" s="27">
         <v>11</v>
       </c>
-      <c r="Q8" s="60">
+      <c r="Q8" s="27">
         <v>12</v>
       </c>
-      <c r="R8" s="60">
+      <c r="R8" s="27">
         <v>13</v>
       </c>
-      <c r="S8" s="60">
+      <c r="S8" s="27">
         <v>14</v>
       </c>
-      <c r="T8" s="60">
+      <c r="T8" s="27">
         <v>15</v>
       </c>
-      <c r="U8" s="60">
+      <c r="U8" s="27">
         <v>16</v>
       </c>
-      <c r="V8" s="60">
+      <c r="V8" s="27">
         <v>17</v>
       </c>
-      <c r="W8" s="60">
+      <c r="W8" s="27">
         <v>18</v>
       </c>
-      <c r="X8" s="60">
+      <c r="X8" s="27">
         <v>19</v>
       </c>
-      <c r="Y8" s="60">
+      <c r="Y8" s="27">
         <v>20</v>
       </c>
-      <c r="Z8" s="60">
+      <c r="Z8" s="27">
         <v>21</v>
       </c>
-      <c r="AA8" s="60">
+      <c r="AA8" s="27">
         <v>22</v>
       </c>
-      <c r="AB8" s="60">
+      <c r="AB8" s="27">
         <v>23</v>
       </c>
-      <c r="AC8" s="60">
+      <c r="AC8" s="27">
         <v>24</v>
       </c>
-      <c r="AD8" s="60">
+      <c r="AD8" s="27">
         <v>25</v>
       </c>
-      <c r="AE8" s="60">
+      <c r="AE8" s="27">
         <v>26</v>
       </c>
-      <c r="AF8" s="60">
+      <c r="AF8" s="27">
         <v>27</v>
       </c>
-      <c r="AG8" s="60">
+      <c r="AG8" s="27">
         <v>28</v>
       </c>
-      <c r="AH8" s="60">
+      <c r="AH8" s="27">
         <v>29</v>
       </c>
-      <c r="AI8" s="60">
+      <c r="AI8" s="27">
         <v>30</v>
       </c>
-      <c r="AJ8" s="60">
+      <c r="AJ8" s="27">
         <v>31</v>
       </c>
-      <c r="AK8" s="60">
+      <c r="AK8" s="27">
         <v>32</v>
       </c>
-      <c r="AL8" s="60">
+      <c r="AL8" s="27">
         <v>33</v>
       </c>
-      <c r="AM8" s="60">
+      <c r="AM8" s="27">
         <v>34</v>
       </c>
-      <c r="AN8" s="60">
+      <c r="AN8" s="27">
         <v>35</v>
       </c>
-      <c r="AO8" s="60">
+      <c r="AO8" s="27">
         <v>36</v>
       </c>
-      <c r="AP8" s="60">
+      <c r="AP8" s="27">
         <v>37</v>
       </c>
-      <c r="AQ8" s="60">
+      <c r="AQ8" s="27">
         <v>38</v>
       </c>
-      <c r="AR8" s="60">
+      <c r="AR8" s="27">
         <v>39</v>
       </c>
-      <c r="AS8" s="60">
+      <c r="AS8" s="27">
         <v>40</v>
       </c>
-      <c r="AT8" s="60">
+      <c r="AT8" s="27">
         <v>41</v>
       </c>
-      <c r="AU8" s="60">
+      <c r="AU8" s="27">
         <v>42</v>
       </c>
-      <c r="AV8" s="60">
+      <c r="AV8" s="27">
         <v>43</v>
       </c>
-      <c r="AW8" s="60">
+      <c r="AW8" s="27">
         <v>44</v>
       </c>
-      <c r="AX8" s="60">
+      <c r="AX8" s="27">
         <v>45</v>
       </c>
-      <c r="AY8" s="60">
+      <c r="AY8" s="27">
         <v>46</v>
       </c>
-      <c r="AZ8" s="60">
+      <c r="AZ8" s="27">
         <v>47</v>
       </c>
-      <c r="BA8" s="60">
+      <c r="BA8" s="27">
         <v>48</v>
       </c>
-      <c r="BB8" s="60">
+      <c r="BB8" s="27">
         <v>49</v>
       </c>
-      <c r="BC8" s="60">
+      <c r="BC8" s="27">
         <v>50</v>
       </c>
-      <c r="BD8" s="60">
+      <c r="BD8" s="27">
         <v>51</v>
       </c>
-      <c r="BE8" s="60">
+      <c r="BE8" s="27">
         <v>52</v>
       </c>
-      <c r="BF8" s="60">
+      <c r="BF8" s="27">
         <v>53</v>
       </c>
-      <c r="BG8" s="60">
+      <c r="BG8" s="27">
         <v>54</v>
       </c>
-      <c r="BH8" s="60">
+      <c r="BH8" s="27">
         <v>55</v>
       </c>
-      <c r="BI8" s="60">
+      <c r="BI8" s="27">
         <v>56</v>
       </c>
-      <c r="BJ8" s="60">
+      <c r="BJ8" s="27">
         <v>57</v>
       </c>
-      <c r="BK8" s="60">
+      <c r="BK8" s="27">
         <v>58</v>
       </c>
-      <c r="BL8" s="60">
+      <c r="BL8" s="27">
         <v>59</v>
       </c>
-      <c r="BM8" s="60">
+      <c r="BM8" s="27">
         <v>60</v>
       </c>
-      <c r="BN8" s="60">
+      <c r="BN8" s="27">
         <v>61</v>
       </c>
-      <c r="BO8" s="60">
+      <c r="BO8" s="27">
         <v>62</v>
       </c>
-      <c r="BP8" s="60">
+      <c r="BP8" s="27">
         <v>63</v>
       </c>
-      <c r="BQ8" s="60">
+      <c r="BQ8" s="27">
         <v>64</v>
       </c>
-      <c r="BR8" s="60">
+      <c r="BR8" s="27">
         <v>65</v>
       </c>
-      <c r="BS8" s="60">
+      <c r="BS8" s="27">
         <v>66</v>
       </c>
-      <c r="BT8" s="60">
+      <c r="BT8" s="27">
         <v>67</v>
       </c>
-      <c r="BU8" s="60">
+      <c r="BU8" s="27">
         <v>68</v>
       </c>
-      <c r="BV8" s="60">
+      <c r="BV8" s="27">
         <v>69</v>
       </c>
-      <c r="BW8" s="60">
+      <c r="BW8" s="27">
         <v>70</v>
       </c>
-      <c r="BX8" s="60">
+      <c r="BX8" s="27">
         <v>71</v>
       </c>
-      <c r="BY8" s="60">
+      <c r="BY8" s="27">
         <v>72</v>
       </c>
-      <c r="BZ8" s="60">
+      <c r="BZ8" s="27">
         <v>73</v>
       </c>
-      <c r="CA8" s="60">
+      <c r="CA8" s="27">
         <v>74</v>
       </c>
-      <c r="CB8" s="60">
+      <c r="CB8" s="27">
         <v>75</v>
       </c>
-      <c r="CC8" s="60">
+      <c r="CC8" s="27">
         <v>76</v>
       </c>
-      <c r="CD8" s="60">
+      <c r="CD8" s="27">
         <v>77</v>
       </c>
-      <c r="CE8" s="60">
+      <c r="CE8" s="27">
         <v>78</v>
       </c>
-      <c r="CF8" s="60">
+      <c r="CF8" s="27">
         <v>79</v>
       </c>
-      <c r="CG8" s="60">
+      <c r="CG8" s="27">
         <v>80</v>
       </c>
-      <c r="CH8" s="60">
+      <c r="CH8" s="27">
         <v>81</v>
       </c>
-      <c r="CI8" s="60">
+      <c r="CI8" s="27">
         <v>82</v>
       </c>
-      <c r="CJ8" s="60">
+      <c r="CJ8" s="27">
         <v>83</v>
       </c>
-      <c r="CK8" s="60">
+      <c r="CK8" s="27">
         <v>84</v>
       </c>
-      <c r="CL8" s="60">
+      <c r="CL8" s="27">
         <v>85</v>
       </c>
-      <c r="CM8" s="60">
+      <c r="CM8" s="27">
         <v>86</v>
       </c>
-      <c r="CN8" s="60">
+      <c r="CN8" s="27">
         <v>87</v>
       </c>
-      <c r="CO8" s="60">
+      <c r="CO8" s="27">
         <v>88</v>
       </c>
-      <c r="CP8" s="60">
+      <c r="CP8" s="27">
         <v>89</v>
       </c>
-      <c r="CQ8" s="60">
+      <c r="CQ8" s="27">
         <v>90</v>
       </c>
-      <c r="CR8" s="60">
+      <c r="CR8" s="27">
         <v>91</v>
       </c>
-      <c r="CS8" s="60">
+      <c r="CS8" s="27">
         <v>92</v>
       </c>
-      <c r="CT8" s="60">
+      <c r="CT8" s="27">
         <v>93</v>
       </c>
-      <c r="CU8" s="60">
+      <c r="CU8" s="27">
         <v>94</v>
       </c>
-      <c r="CV8" s="60">
+      <c r="CV8" s="27">
         <v>95</v>
       </c>
-      <c r="CW8" s="60">
+      <c r="CW8" s="27">
         <v>96</v>
       </c>
-      <c r="CX8" s="60">
+      <c r="CX8" s="27">
         <v>97</v>
       </c>
-      <c r="CY8" s="60">
+      <c r="CY8" s="27">
         <v>98</v>
       </c>
-      <c r="CZ8" s="60">
+      <c r="CZ8" s="27">
         <v>99</v>
       </c>
-      <c r="DA8" s="60">
+      <c r="DA8" s="27">
         <v>100</v>
       </c>
-      <c r="DB8" s="60">
+      <c r="DB8" s="27">
         <v>101</v>
       </c>
-      <c r="DC8" s="60">
+      <c r="DC8" s="27">
         <v>102</v>
       </c>
-      <c r="DD8" s="60">
+      <c r="DD8" s="27">
         <v>103</v>
       </c>
-      <c r="DE8" s="60">
+      <c r="DE8" s="27">
         <v>104</v>
       </c>
-      <c r="DF8" s="60">
+      <c r="DF8" s="27">
         <v>105</v>
       </c>
-      <c r="DG8" s="60">
+      <c r="DG8" s="27">
         <v>106</v>
       </c>
-      <c r="DH8" s="60">
+      <c r="DH8" s="27">
         <v>107</v>
       </c>
-      <c r="DI8" s="60">
+      <c r="DI8" s="27">
         <v>108</v>
       </c>
-      <c r="DJ8" s="60">
+      <c r="DJ8" s="27">
         <v>109</v>
       </c>
-      <c r="DK8" s="60">
+      <c r="DK8" s="27">
         <v>110</v>
       </c>
-      <c r="DL8" s="60">
+      <c r="DL8" s="27">
         <v>111</v>
       </c>
-      <c r="DM8" s="60">
+      <c r="DM8" s="27">
         <v>112</v>
       </c>
-      <c r="DN8" s="60">
+      <c r="DN8" s="27">
         <v>113</v>
       </c>
-      <c r="DO8" s="60">
+      <c r="DO8" s="27">
         <v>114</v>
       </c>
-      <c r="DP8" s="60">
+      <c r="DP8" s="27">
         <v>115</v>
       </c>
-      <c r="DQ8" s="60">
+      <c r="DQ8" s="27">
         <v>116</v>
       </c>
-      <c r="DR8" s="60">
+      <c r="DR8" s="27">
         <v>117</v>
       </c>
-      <c r="DS8" s="60">
+      <c r="DS8" s="27">
         <v>118</v>
       </c>
-      <c r="DT8" s="60">
+      <c r="DT8" s="27">
         <v>119</v>
       </c>
-      <c r="DU8" s="60">
+      <c r="DU8" s="27">
         <v>120</v>
       </c>
-      <c r="DV8" s="60">
+      <c r="DV8" s="27">
         <v>121</v>
       </c>
-      <c r="DW8" s="60">
+      <c r="DW8" s="27">
         <v>122</v>
       </c>
-      <c r="DX8" s="60">
+      <c r="DX8" s="27">
         <v>123</v>
       </c>
-      <c r="DY8" s="60">
+      <c r="DY8" s="27">
         <v>124</v>
       </c>
-      <c r="DZ8" s="60">
+      <c r="DZ8" s="27">
         <v>125</v>
       </c>
-      <c r="EA8" s="60">
+      <c r="EA8" s="27">
         <v>126</v>
       </c>
-      <c r="EB8" s="60">
+      <c r="EB8" s="27">
         <v>127</v>
       </c>
-      <c r="EC8" s="60">
+      <c r="EC8" s="27">
         <v>128</v>
       </c>
-      <c r="ED8" s="60">
+      <c r="ED8" s="27">
         <v>129</v>
       </c>
-      <c r="EE8" s="60">
+      <c r="EE8" s="27">
         <v>130</v>
       </c>
-      <c r="EF8" s="60">
+      <c r="EF8" s="27">
         <v>131</v>
       </c>
-      <c r="EG8" s="60">
+      <c r="EG8" s="27">
         <v>132</v>
       </c>
-      <c r="EH8" s="60">
+      <c r="EH8" s="27">
         <v>133</v>
       </c>
-      <c r="EI8" s="60">
+      <c r="EI8" s="27">
         <v>134</v>
       </c>
-      <c r="EJ8" s="60">
+      <c r="EJ8" s="27">
         <v>135</v>
       </c>
-      <c r="EK8" s="60">
+      <c r="EK8" s="27">
         <v>136</v>
       </c>
-      <c r="EL8" s="60">
+      <c r="EL8" s="27">
         <v>137</v>
       </c>
-      <c r="EM8" s="60">
+      <c r="EM8" s="27">
         <v>138</v>
       </c>
-      <c r="EN8" s="60">
+      <c r="EN8" s="27">
         <v>139</v>
       </c>
-      <c r="EO8" s="60">
+      <c r="EO8" s="27">
         <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="62" t="s">
+      <c r="A9" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="64" t="s">
+      <c r="C9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="63"/>
+      <c r="D9" s="37"/>
       <c r="E9" s="8"/>
-      <c r="F9" s="61"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="61"/>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="61"/>
-      <c r="N9" s="61"/>
-      <c r="O9" s="61"/>
-      <c r="P9" s="61"/>
-      <c r="Q9" s="61"/>
-      <c r="R9" s="61"/>
-      <c r="S9" s="61"/>
-      <c r="T9" s="61"/>
-      <c r="U9" s="61"/>
-      <c r="V9" s="61"/>
-      <c r="W9" s="61"/>
-      <c r="X9" s="61"/>
-      <c r="Y9" s="61"/>
-      <c r="Z9" s="61"/>
-      <c r="AA9" s="61"/>
-      <c r="AB9" s="61"/>
-      <c r="AC9" s="61"/>
-      <c r="AD9" s="61"/>
-      <c r="AE9" s="61"/>
-      <c r="AF9" s="61"/>
-      <c r="AG9" s="61"/>
-      <c r="AH9" s="61"/>
-      <c r="AI9" s="61"/>
-      <c r="AJ9" s="61"/>
-      <c r="AK9" s="61"/>
-      <c r="AL9" s="61"/>
-      <c r="AM9" s="61"/>
-      <c r="AN9" s="61"/>
-      <c r="AO9" s="61"/>
-      <c r="AP9" s="61"/>
-      <c r="AQ9" s="61"/>
-      <c r="AR9" s="61"/>
-      <c r="AS9" s="61"/>
-      <c r="AT9" s="61"/>
-      <c r="AU9" s="61"/>
-      <c r="AV9" s="61"/>
-      <c r="AW9" s="61"/>
-      <c r="AX9" s="61"/>
-      <c r="AY9" s="61"/>
-      <c r="AZ9" s="61"/>
-      <c r="BA9" s="61"/>
-      <c r="BB9" s="61"/>
-      <c r="BC9" s="61"/>
-      <c r="BD9" s="61"/>
-      <c r="BE9" s="61"/>
-      <c r="BF9" s="61"/>
-      <c r="BG9" s="61"/>
-      <c r="BH9" s="61"/>
-      <c r="BI9" s="61"/>
-      <c r="BJ9" s="61"/>
-      <c r="BK9" s="61"/>
-      <c r="BL9" s="61"/>
-      <c r="BM9" s="61"/>
-      <c r="BN9" s="61"/>
-      <c r="BO9" s="61"/>
-      <c r="BP9" s="61"/>
-      <c r="BQ9" s="61"/>
-      <c r="BR9" s="61"/>
-      <c r="BS9" s="61"/>
-      <c r="BT9" s="61"/>
-      <c r="BU9" s="61"/>
-      <c r="BV9" s="61"/>
-      <c r="BW9" s="61"/>
-      <c r="BX9" s="61"/>
-      <c r="BY9" s="61"/>
-      <c r="BZ9" s="61"/>
-      <c r="CA9" s="61"/>
-      <c r="CB9" s="61"/>
-      <c r="CC9" s="61"/>
-      <c r="CD9" s="61"/>
-      <c r="CE9" s="61"/>
-      <c r="CF9" s="61"/>
-      <c r="CG9" s="61"/>
-      <c r="CH9" s="61"/>
-      <c r="CI9" s="61"/>
-      <c r="CJ9" s="61"/>
-      <c r="CK9" s="61"/>
-      <c r="CL9" s="61"/>
-      <c r="CM9" s="61"/>
-      <c r="CN9" s="61"/>
-      <c r="CO9" s="61"/>
-      <c r="CP9" s="61"/>
-      <c r="CQ9" s="61"/>
-      <c r="CR9" s="61"/>
-      <c r="CS9" s="61"/>
-      <c r="CT9" s="61"/>
-      <c r="CU9" s="61"/>
-      <c r="CV9" s="61"/>
-      <c r="CW9" s="61"/>
-      <c r="CX9" s="61"/>
-      <c r="CY9" s="61"/>
-      <c r="CZ9" s="61"/>
-      <c r="DA9" s="61"/>
-      <c r="DB9" s="61"/>
-      <c r="DC9" s="61"/>
-      <c r="DD9" s="61"/>
-      <c r="DE9" s="61"/>
-      <c r="DF9" s="61"/>
-      <c r="DG9" s="61"/>
-      <c r="DH9" s="61"/>
-      <c r="DI9" s="61"/>
-      <c r="DJ9" s="61"/>
-      <c r="DK9" s="61"/>
-      <c r="DL9" s="61"/>
-      <c r="DM9" s="61"/>
-      <c r="DN9" s="61"/>
-      <c r="DO9" s="61"/>
-      <c r="DP9" s="61"/>
-      <c r="DQ9" s="61"/>
-      <c r="DR9" s="61"/>
-      <c r="DS9" s="61"/>
-      <c r="DT9" s="61"/>
-      <c r="DU9" s="61"/>
-      <c r="DV9" s="61"/>
-      <c r="DW9" s="61"/>
-      <c r="DX9" s="61"/>
-      <c r="DY9" s="61"/>
-      <c r="DZ9" s="61"/>
-      <c r="EA9" s="61"/>
-      <c r="EB9" s="61"/>
-      <c r="EC9" s="61"/>
-      <c r="ED9" s="61"/>
-      <c r="EE9" s="61"/>
-      <c r="EF9" s="61"/>
-      <c r="EG9" s="61"/>
-      <c r="EH9" s="61"/>
-      <c r="EI9" s="61"/>
-      <c r="EJ9" s="61"/>
-      <c r="EK9" s="61"/>
-      <c r="EL9" s="61"/>
-      <c r="EM9" s="61"/>
-      <c r="EN9" s="61"/>
-      <c r="EO9" s="61"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="28"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
+      <c r="Q9" s="28"/>
+      <c r="R9" s="28"/>
+      <c r="S9" s="28"/>
+      <c r="T9" s="28"/>
+      <c r="U9" s="28"/>
+      <c r="V9" s="28"/>
+      <c r="W9" s="28"/>
+      <c r="X9" s="28"/>
+      <c r="Y9" s="28"/>
+      <c r="Z9" s="28"/>
+      <c r="AA9" s="28"/>
+      <c r="AB9" s="28"/>
+      <c r="AC9" s="28"/>
+      <c r="AD9" s="28"/>
+      <c r="AE9" s="28"/>
+      <c r="AF9" s="28"/>
+      <c r="AG9" s="28"/>
+      <c r="AH9" s="28"/>
+      <c r="AI9" s="28"/>
+      <c r="AJ9" s="28"/>
+      <c r="AK9" s="28"/>
+      <c r="AL9" s="28"/>
+      <c r="AM9" s="28"/>
+      <c r="AN9" s="28"/>
+      <c r="AO9" s="28"/>
+      <c r="AP9" s="28"/>
+      <c r="AQ9" s="28"/>
+      <c r="AR9" s="28"/>
+      <c r="AS9" s="28"/>
+      <c r="AT9" s="28"/>
+      <c r="AU9" s="28"/>
+      <c r="AV9" s="28"/>
+      <c r="AW9" s="28"/>
+      <c r="AX9" s="28"/>
+      <c r="AY9" s="28"/>
+      <c r="AZ9" s="28"/>
+      <c r="BA9" s="28"/>
+      <c r="BB9" s="28"/>
+      <c r="BC9" s="28"/>
+      <c r="BD9" s="28"/>
+      <c r="BE9" s="28"/>
+      <c r="BF9" s="28"/>
+      <c r="BG9" s="28"/>
+      <c r="BH9" s="28"/>
+      <c r="BI9" s="28"/>
+      <c r="BJ9" s="28"/>
+      <c r="BK9" s="28"/>
+      <c r="BL9" s="28"/>
+      <c r="BM9" s="28"/>
+      <c r="BN9" s="28"/>
+      <c r="BO9" s="28"/>
+      <c r="BP9" s="28"/>
+      <c r="BQ9" s="28"/>
+      <c r="BR9" s="28"/>
+      <c r="BS9" s="28"/>
+      <c r="BT9" s="28"/>
+      <c r="BU9" s="28"/>
+      <c r="BV9" s="28"/>
+      <c r="BW9" s="28"/>
+      <c r="BX9" s="28"/>
+      <c r="BY9" s="28"/>
+      <c r="BZ9" s="28"/>
+      <c r="CA9" s="28"/>
+      <c r="CB9" s="28"/>
+      <c r="CC9" s="28"/>
+      <c r="CD9" s="28"/>
+      <c r="CE9" s="28"/>
+      <c r="CF9" s="28"/>
+      <c r="CG9" s="28"/>
+      <c r="CH9" s="28"/>
+      <c r="CI9" s="28"/>
+      <c r="CJ9" s="28"/>
+      <c r="CK9" s="28"/>
+      <c r="CL9" s="28"/>
+      <c r="CM9" s="28"/>
+      <c r="CN9" s="28"/>
+      <c r="CO9" s="28"/>
+      <c r="CP9" s="28"/>
+      <c r="CQ9" s="28"/>
+      <c r="CR9" s="28"/>
+      <c r="CS9" s="28"/>
+      <c r="CT9" s="28"/>
+      <c r="CU9" s="28"/>
+      <c r="CV9" s="28"/>
+      <c r="CW9" s="28"/>
+      <c r="CX9" s="28"/>
+      <c r="CY9" s="28"/>
+      <c r="CZ9" s="28"/>
+      <c r="DA9" s="28"/>
+      <c r="DB9" s="28"/>
+      <c r="DC9" s="28"/>
+      <c r="DD9" s="28"/>
+      <c r="DE9" s="28"/>
+      <c r="DF9" s="28"/>
+      <c r="DG9" s="28"/>
+      <c r="DH9" s="28"/>
+      <c r="DI9" s="28"/>
+      <c r="DJ9" s="28"/>
+      <c r="DK9" s="28"/>
+      <c r="DL9" s="28"/>
+      <c r="DM9" s="28"/>
+      <c r="DN9" s="28"/>
+      <c r="DO9" s="28"/>
+      <c r="DP9" s="28"/>
+      <c r="DQ9" s="28"/>
+      <c r="DR9" s="28"/>
+      <c r="DS9" s="28"/>
+      <c r="DT9" s="28"/>
+      <c r="DU9" s="28"/>
+      <c r="DV9" s="28"/>
+      <c r="DW9" s="28"/>
+      <c r="DX9" s="28"/>
+      <c r="DY9" s="28"/>
+      <c r="DZ9" s="28"/>
+      <c r="EA9" s="28"/>
+      <c r="EB9" s="28"/>
+      <c r="EC9" s="28"/>
+      <c r="ED9" s="28"/>
+      <c r="EE9" s="28"/>
+      <c r="EF9" s="28"/>
+      <c r="EG9" s="28"/>
+      <c r="EH9" s="28"/>
+      <c r="EI9" s="28"/>
+      <c r="EJ9" s="28"/>
+      <c r="EK9" s="28"/>
+      <c r="EL9" s="28"/>
+      <c r="EM9" s="28"/>
+      <c r="EN9" s="28"/>
+      <c r="EO9" s="28"/>
     </row>
     <row r="10" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="62"/>
-      <c r="B10" s="63"/>
+      <c r="A10" s="36"/>
+      <c r="B10" s="37"/>
       <c r="C10" s="9"/>
       <c r="D10" s="7" t="s">
         <v>19</v>
@@ -3202,7 +3209,7 @@
       <c r="EN10" s="11"/>
       <c r="EO10" s="11"/>
     </row>
-    <row r="11" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12">
         <v>1</v>
       </c>
@@ -3358,7 +3365,7 @@
       <c r="EN11" s="11"/>
       <c r="EO11" s="11"/>
     </row>
-    <row r="12" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12">
         <v>2</v>
       </c>
@@ -3556,7 +3563,7 @@
       <c r="EN12" s="11"/>
       <c r="EO12" s="11"/>
     </row>
-    <row r="13" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
         <v>3</v>
       </c>
@@ -3782,7 +3789,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <v>4</v>
       </c>
@@ -3978,7 +3985,7 @@
       <c r="EN14" s="11"/>
       <c r="EO14" s="11"/>
     </row>
-    <row r="15" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12">
         <v>5</v>
       </c>
@@ -4178,7 +4185,7 @@
       <c r="EN15" s="11"/>
       <c r="EO15" s="11"/>
     </row>
-    <row r="16" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:150" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <v>6</v>
       </c>
@@ -4368,7 +4375,7 @@
       <c r="EN16" s="11"/>
       <c r="EO16" s="11"/>
     </row>
-    <row r="17" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <v>7</v>
       </c>
@@ -4478,115 +4485,115 @@
       <c r="AN17" s="11">
         <v>0</v>
       </c>
-      <c r="AO17" s="23" t="s">
+      <c r="AO17" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="AP17" s="24"/>
-      <c r="AQ17" s="24"/>
-      <c r="AR17" s="24"/>
-      <c r="AS17" s="24"/>
-      <c r="AT17" s="24"/>
-      <c r="AU17" s="24"/>
-      <c r="AV17" s="24"/>
-      <c r="AW17" s="24"/>
-      <c r="AX17" s="24"/>
-      <c r="AY17" s="24"/>
-      <c r="AZ17" s="24"/>
-      <c r="BA17" s="24"/>
-      <c r="BB17" s="24"/>
-      <c r="BC17" s="24"/>
-      <c r="BD17" s="24"/>
-      <c r="BE17" s="24"/>
-      <c r="BF17" s="24"/>
-      <c r="BG17" s="24"/>
-      <c r="BH17" s="24"/>
-      <c r="BI17" s="24"/>
-      <c r="BJ17" s="24"/>
-      <c r="BK17" s="24"/>
-      <c r="BL17" s="24"/>
-      <c r="BM17" s="24"/>
-      <c r="BN17" s="24"/>
-      <c r="BO17" s="24"/>
-      <c r="BP17" s="24"/>
-      <c r="BQ17" s="24"/>
-      <c r="BR17" s="24"/>
-      <c r="BS17" s="24"/>
-      <c r="BT17" s="24"/>
-      <c r="BU17" s="24"/>
-      <c r="BV17" s="24"/>
-      <c r="BW17" s="24"/>
-      <c r="BX17" s="24"/>
-      <c r="BY17" s="24"/>
-      <c r="BZ17" s="24"/>
-      <c r="CA17" s="24"/>
-      <c r="CB17" s="24"/>
-      <c r="CC17" s="24"/>
-      <c r="CD17" s="24"/>
-      <c r="CE17" s="24"/>
-      <c r="CF17" s="24"/>
-      <c r="CG17" s="24"/>
-      <c r="CH17" s="24"/>
-      <c r="CI17" s="24"/>
-      <c r="CJ17" s="24"/>
-      <c r="CK17" s="24"/>
-      <c r="CL17" s="24"/>
-      <c r="CM17" s="24"/>
-      <c r="CN17" s="24"/>
-      <c r="CO17" s="24"/>
-      <c r="CP17" s="24"/>
-      <c r="CQ17" s="24"/>
-      <c r="CR17" s="24"/>
-      <c r="CS17" s="24"/>
-      <c r="CT17" s="24"/>
-      <c r="CU17" s="24"/>
-      <c r="CV17" s="24"/>
-      <c r="CW17" s="24"/>
-      <c r="CX17" s="24"/>
-      <c r="CY17" s="24"/>
-      <c r="CZ17" s="24"/>
-      <c r="DA17" s="24"/>
-      <c r="DB17" s="24"/>
-      <c r="DC17" s="24"/>
-      <c r="DD17" s="24"/>
-      <c r="DE17" s="24"/>
-      <c r="DF17" s="24"/>
-      <c r="DG17" s="24"/>
-      <c r="DH17" s="24"/>
-      <c r="DI17" s="24"/>
-      <c r="DJ17" s="24"/>
-      <c r="DK17" s="24"/>
-      <c r="DL17" s="24"/>
-      <c r="DM17" s="24"/>
-      <c r="DN17" s="24"/>
-      <c r="DO17" s="24"/>
-      <c r="DP17" s="24"/>
-      <c r="DQ17" s="24"/>
-      <c r="DR17" s="24"/>
-      <c r="DS17" s="24"/>
-      <c r="DT17" s="24"/>
-      <c r="DU17" s="24"/>
-      <c r="DV17" s="24"/>
-      <c r="DW17" s="24"/>
-      <c r="DX17" s="24"/>
-      <c r="DY17" s="24"/>
-      <c r="DZ17" s="24"/>
-      <c r="EA17" s="24"/>
-      <c r="EB17" s="24"/>
-      <c r="EC17" s="24"/>
-      <c r="ED17" s="24"/>
-      <c r="EE17" s="24"/>
-      <c r="EF17" s="24"/>
-      <c r="EG17" s="24"/>
-      <c r="EH17" s="24"/>
-      <c r="EI17" s="24"/>
-      <c r="EJ17" s="24"/>
-      <c r="EK17" s="24"/>
-      <c r="EL17" s="24"/>
-      <c r="EM17" s="24"/>
-      <c r="EN17" s="24"/>
-      <c r="EO17" s="25"/>
+      <c r="AP17" s="54"/>
+      <c r="AQ17" s="54"/>
+      <c r="AR17" s="54"/>
+      <c r="AS17" s="54"/>
+      <c r="AT17" s="54"/>
+      <c r="AU17" s="54"/>
+      <c r="AV17" s="54"/>
+      <c r="AW17" s="54"/>
+      <c r="AX17" s="54"/>
+      <c r="AY17" s="54"/>
+      <c r="AZ17" s="54"/>
+      <c r="BA17" s="54"/>
+      <c r="BB17" s="54"/>
+      <c r="BC17" s="54"/>
+      <c r="BD17" s="54"/>
+      <c r="BE17" s="54"/>
+      <c r="BF17" s="54"/>
+      <c r="BG17" s="54"/>
+      <c r="BH17" s="54"/>
+      <c r="BI17" s="54"/>
+      <c r="BJ17" s="54"/>
+      <c r="BK17" s="54"/>
+      <c r="BL17" s="54"/>
+      <c r="BM17" s="54"/>
+      <c r="BN17" s="54"/>
+      <c r="BO17" s="54"/>
+      <c r="BP17" s="54"/>
+      <c r="BQ17" s="54"/>
+      <c r="BR17" s="54"/>
+      <c r="BS17" s="54"/>
+      <c r="BT17" s="54"/>
+      <c r="BU17" s="54"/>
+      <c r="BV17" s="54"/>
+      <c r="BW17" s="54"/>
+      <c r="BX17" s="54"/>
+      <c r="BY17" s="54"/>
+      <c r="BZ17" s="54"/>
+      <c r="CA17" s="54"/>
+      <c r="CB17" s="54"/>
+      <c r="CC17" s="54"/>
+      <c r="CD17" s="54"/>
+      <c r="CE17" s="54"/>
+      <c r="CF17" s="54"/>
+      <c r="CG17" s="54"/>
+      <c r="CH17" s="54"/>
+      <c r="CI17" s="54"/>
+      <c r="CJ17" s="54"/>
+      <c r="CK17" s="54"/>
+      <c r="CL17" s="54"/>
+      <c r="CM17" s="54"/>
+      <c r="CN17" s="54"/>
+      <c r="CO17" s="54"/>
+      <c r="CP17" s="54"/>
+      <c r="CQ17" s="54"/>
+      <c r="CR17" s="54"/>
+      <c r="CS17" s="54"/>
+      <c r="CT17" s="54"/>
+      <c r="CU17" s="54"/>
+      <c r="CV17" s="54"/>
+      <c r="CW17" s="54"/>
+      <c r="CX17" s="54"/>
+      <c r="CY17" s="54"/>
+      <c r="CZ17" s="54"/>
+      <c r="DA17" s="54"/>
+      <c r="DB17" s="54"/>
+      <c r="DC17" s="54"/>
+      <c r="DD17" s="54"/>
+      <c r="DE17" s="54"/>
+      <c r="DF17" s="54"/>
+      <c r="DG17" s="54"/>
+      <c r="DH17" s="54"/>
+      <c r="DI17" s="54"/>
+      <c r="DJ17" s="54"/>
+      <c r="DK17" s="54"/>
+      <c r="DL17" s="54"/>
+      <c r="DM17" s="54"/>
+      <c r="DN17" s="54"/>
+      <c r="DO17" s="54"/>
+      <c r="DP17" s="54"/>
+      <c r="DQ17" s="54"/>
+      <c r="DR17" s="54"/>
+      <c r="DS17" s="54"/>
+      <c r="DT17" s="54"/>
+      <c r="DU17" s="54"/>
+      <c r="DV17" s="54"/>
+      <c r="DW17" s="54"/>
+      <c r="DX17" s="54"/>
+      <c r="DY17" s="54"/>
+      <c r="DZ17" s="54"/>
+      <c r="EA17" s="54"/>
+      <c r="EB17" s="54"/>
+      <c r="EC17" s="54"/>
+      <c r="ED17" s="54"/>
+      <c r="EE17" s="54"/>
+      <c r="EF17" s="54"/>
+      <c r="EG17" s="54"/>
+      <c r="EH17" s="54"/>
+      <c r="EI17" s="54"/>
+      <c r="EJ17" s="54"/>
+      <c r="EK17" s="54"/>
+      <c r="EL17" s="54"/>
+      <c r="EM17" s="54"/>
+      <c r="EN17" s="54"/>
+      <c r="EO17" s="55"/>
     </row>
-    <row r="18" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12">
         <v>8</v>
       </c>
@@ -4766,7 +4773,7 @@
       <c r="EN18" s="11"/>
       <c r="EO18" s="11"/>
     </row>
-    <row r="19" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12">
         <v>9</v>
       </c>
@@ -4966,7 +4973,7 @@
       <c r="EN19" s="11"/>
       <c r="EO19" s="11"/>
     </row>
-    <row r="20" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12">
         <v>10</v>
       </c>
@@ -5136,7 +5143,7 @@
       <c r="EN20" s="11"/>
       <c r="EO20" s="11"/>
     </row>
-    <row r="21" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
         <v>11</v>
       </c>
@@ -5420,7 +5427,7 @@
       <c r="EN21" s="11"/>
       <c r="EO21" s="11"/>
     </row>
-    <row r="22" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12">
         <v>12</v>
       </c>
@@ -5636,7 +5643,7 @@
       <c r="EN22" s="11"/>
       <c r="EO22" s="11"/>
     </row>
-    <row r="23" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12">
         <v>13</v>
       </c>
@@ -5924,7 +5931,7 @@
       <c r="EN23" s="11"/>
       <c r="EO23" s="11"/>
     </row>
-    <row r="24" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12">
         <v>14</v>
       </c>
@@ -6134,7 +6141,7 @@
       <c r="EN24" s="11"/>
       <c r="EO24" s="11"/>
     </row>
-    <row r="25" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12">
         <v>15</v>
       </c>
@@ -6360,7 +6367,7 @@
       <c r="EN25" s="11"/>
       <c r="EO25" s="11"/>
     </row>
-    <row r="26" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12">
         <v>16</v>
       </c>
@@ -6576,7 +6583,7 @@
       <c r="EN26" s="11"/>
       <c r="EO26" s="11"/>
     </row>
-    <row r="27" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
         <v>17</v>
       </c>
@@ -6862,7 +6869,7 @@
       <c r="EN27" s="11"/>
       <c r="EO27" s="11"/>
     </row>
-    <row r="28" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12">
         <v>18</v>
       </c>
@@ -6876,149 +6883,149 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E28" s="65" t="s">
+      <c r="E28" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="F28" s="65"/>
-      <c r="G28" s="65"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="65"/>
-      <c r="J28" s="65"/>
-      <c r="K28" s="65"/>
-      <c r="L28" s="65"/>
-      <c r="M28" s="65"/>
-      <c r="N28" s="65"/>
-      <c r="O28" s="65"/>
-      <c r="P28" s="65"/>
-      <c r="Q28" s="65"/>
-      <c r="R28" s="65"/>
-      <c r="S28" s="65"/>
-      <c r="T28" s="65"/>
-      <c r="U28" s="65"/>
-      <c r="V28" s="65"/>
-      <c r="W28" s="65"/>
-      <c r="X28" s="65"/>
-      <c r="Y28" s="65"/>
-      <c r="Z28" s="65"/>
-      <c r="AA28" s="65"/>
-      <c r="AB28" s="65"/>
-      <c r="AC28" s="65"/>
-      <c r="AD28" s="65"/>
-      <c r="AE28" s="65"/>
-      <c r="AF28" s="65"/>
-      <c r="AG28" s="65"/>
-      <c r="AH28" s="65"/>
-      <c r="AI28" s="65"/>
-      <c r="AJ28" s="65"/>
-      <c r="AK28" s="65"/>
-      <c r="AL28" s="65"/>
-      <c r="AM28" s="65"/>
-      <c r="AN28" s="65"/>
-      <c r="AO28" s="65"/>
-      <c r="AP28" s="65"/>
-      <c r="AQ28" s="65"/>
-      <c r="AR28" s="65"/>
-      <c r="AS28" s="65"/>
-      <c r="AT28" s="65"/>
-      <c r="AU28" s="65"/>
-      <c r="AV28" s="65"/>
-      <c r="AW28" s="65"/>
-      <c r="AX28" s="65"/>
-      <c r="AY28" s="65"/>
-      <c r="AZ28" s="65"/>
-      <c r="BA28" s="65"/>
-      <c r="BB28" s="65"/>
-      <c r="BC28" s="65"/>
-      <c r="BD28" s="65"/>
-      <c r="BE28" s="65"/>
-      <c r="BF28" s="65"/>
-      <c r="BG28" s="65"/>
-      <c r="BH28" s="65"/>
-      <c r="BI28" s="65"/>
-      <c r="BJ28" s="65"/>
-      <c r="BK28" s="65"/>
-      <c r="BL28" s="65"/>
-      <c r="BM28" s="65"/>
-      <c r="BN28" s="65"/>
-      <c r="BO28" s="65"/>
-      <c r="BP28" s="65"/>
-      <c r="BQ28" s="65"/>
-      <c r="BR28" s="65"/>
-      <c r="BS28" s="65"/>
-      <c r="BT28" s="65"/>
-      <c r="BU28" s="65"/>
-      <c r="BV28" s="65"/>
-      <c r="BW28" s="65"/>
-      <c r="BX28" s="65"/>
-      <c r="BY28" s="65"/>
-      <c r="BZ28" s="65"/>
-      <c r="CA28" s="65"/>
-      <c r="CB28" s="65"/>
-      <c r="CC28" s="65"/>
-      <c r="CD28" s="65"/>
-      <c r="CE28" s="65"/>
-      <c r="CF28" s="65"/>
-      <c r="CG28" s="65"/>
-      <c r="CH28" s="65"/>
-      <c r="CI28" s="65"/>
-      <c r="CJ28" s="65"/>
-      <c r="CK28" s="65"/>
-      <c r="CL28" s="65"/>
-      <c r="CM28" s="65"/>
-      <c r="CN28" s="65"/>
-      <c r="CO28" s="65"/>
-      <c r="CP28" s="65"/>
-      <c r="CQ28" s="65"/>
-      <c r="CR28" s="65"/>
-      <c r="CS28" s="65"/>
-      <c r="CT28" s="65"/>
-      <c r="CU28" s="65"/>
-      <c r="CV28" s="65"/>
-      <c r="CW28" s="65"/>
-      <c r="CX28" s="65"/>
-      <c r="CY28" s="65"/>
-      <c r="CZ28" s="65"/>
-      <c r="DA28" s="65"/>
-      <c r="DB28" s="65"/>
-      <c r="DC28" s="65"/>
-      <c r="DD28" s="65"/>
-      <c r="DE28" s="65"/>
-      <c r="DF28" s="65"/>
-      <c r="DG28" s="65"/>
-      <c r="DH28" s="65"/>
-      <c r="DI28" s="65"/>
-      <c r="DJ28" s="65"/>
-      <c r="DK28" s="65"/>
-      <c r="DL28" s="65"/>
-      <c r="DM28" s="65"/>
-      <c r="DN28" s="65"/>
-      <c r="DO28" s="65"/>
-      <c r="DP28" s="65"/>
-      <c r="DQ28" s="65"/>
-      <c r="DR28" s="65"/>
-      <c r="DS28" s="65"/>
-      <c r="DT28" s="65"/>
-      <c r="DU28" s="65"/>
-      <c r="DV28" s="65"/>
-      <c r="DW28" s="65"/>
-      <c r="DX28" s="65"/>
-      <c r="DY28" s="65"/>
-      <c r="DZ28" s="65"/>
-      <c r="EA28" s="65"/>
-      <c r="EB28" s="65"/>
-      <c r="EC28" s="65"/>
-      <c r="ED28" s="65"/>
-      <c r="EE28" s="65"/>
-      <c r="EF28" s="65"/>
-      <c r="EG28" s="65"/>
-      <c r="EH28" s="65"/>
-      <c r="EI28" s="65"/>
-      <c r="EJ28" s="65"/>
-      <c r="EK28" s="65"/>
-      <c r="EL28" s="65"/>
-      <c r="EM28" s="65"/>
-      <c r="EN28" s="65"/>
-      <c r="EO28" s="65"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="29"/>
+      <c r="N28" s="29"/>
+      <c r="O28" s="29"/>
+      <c r="P28" s="29"/>
+      <c r="Q28" s="29"/>
+      <c r="R28" s="29"/>
+      <c r="S28" s="29"/>
+      <c r="T28" s="29"/>
+      <c r="U28" s="29"/>
+      <c r="V28" s="29"/>
+      <c r="W28" s="29"/>
+      <c r="X28" s="29"/>
+      <c r="Y28" s="29"/>
+      <c r="Z28" s="29"/>
+      <c r="AA28" s="29"/>
+      <c r="AB28" s="29"/>
+      <c r="AC28" s="29"/>
+      <c r="AD28" s="29"/>
+      <c r="AE28" s="29"/>
+      <c r="AF28" s="29"/>
+      <c r="AG28" s="29"/>
+      <c r="AH28" s="29"/>
+      <c r="AI28" s="29"/>
+      <c r="AJ28" s="29"/>
+      <c r="AK28" s="29"/>
+      <c r="AL28" s="29"/>
+      <c r="AM28" s="29"/>
+      <c r="AN28" s="29"/>
+      <c r="AO28" s="29"/>
+      <c r="AP28" s="29"/>
+      <c r="AQ28" s="29"/>
+      <c r="AR28" s="29"/>
+      <c r="AS28" s="29"/>
+      <c r="AT28" s="29"/>
+      <c r="AU28" s="29"/>
+      <c r="AV28" s="29"/>
+      <c r="AW28" s="29"/>
+      <c r="AX28" s="29"/>
+      <c r="AY28" s="29"/>
+      <c r="AZ28" s="29"/>
+      <c r="BA28" s="29"/>
+      <c r="BB28" s="29"/>
+      <c r="BC28" s="29"/>
+      <c r="BD28" s="29"/>
+      <c r="BE28" s="29"/>
+      <c r="BF28" s="29"/>
+      <c r="BG28" s="29"/>
+      <c r="BH28" s="29"/>
+      <c r="BI28" s="29"/>
+      <c r="BJ28" s="29"/>
+      <c r="BK28" s="29"/>
+      <c r="BL28" s="29"/>
+      <c r="BM28" s="29"/>
+      <c r="BN28" s="29"/>
+      <c r="BO28" s="29"/>
+      <c r="BP28" s="29"/>
+      <c r="BQ28" s="29"/>
+      <c r="BR28" s="29"/>
+      <c r="BS28" s="29"/>
+      <c r="BT28" s="29"/>
+      <c r="BU28" s="29"/>
+      <c r="BV28" s="29"/>
+      <c r="BW28" s="29"/>
+      <c r="BX28" s="29"/>
+      <c r="BY28" s="29"/>
+      <c r="BZ28" s="29"/>
+      <c r="CA28" s="29"/>
+      <c r="CB28" s="29"/>
+      <c r="CC28" s="29"/>
+      <c r="CD28" s="29"/>
+      <c r="CE28" s="29"/>
+      <c r="CF28" s="29"/>
+      <c r="CG28" s="29"/>
+      <c r="CH28" s="29"/>
+      <c r="CI28" s="29"/>
+      <c r="CJ28" s="29"/>
+      <c r="CK28" s="29"/>
+      <c r="CL28" s="29"/>
+      <c r="CM28" s="29"/>
+      <c r="CN28" s="29"/>
+      <c r="CO28" s="29"/>
+      <c r="CP28" s="29"/>
+      <c r="CQ28" s="29"/>
+      <c r="CR28" s="29"/>
+      <c r="CS28" s="29"/>
+      <c r="CT28" s="29"/>
+      <c r="CU28" s="29"/>
+      <c r="CV28" s="29"/>
+      <c r="CW28" s="29"/>
+      <c r="CX28" s="29"/>
+      <c r="CY28" s="29"/>
+      <c r="CZ28" s="29"/>
+      <c r="DA28" s="29"/>
+      <c r="DB28" s="29"/>
+      <c r="DC28" s="29"/>
+      <c r="DD28" s="29"/>
+      <c r="DE28" s="29"/>
+      <c r="DF28" s="29"/>
+      <c r="DG28" s="29"/>
+      <c r="DH28" s="29"/>
+      <c r="DI28" s="29"/>
+      <c r="DJ28" s="29"/>
+      <c r="DK28" s="29"/>
+      <c r="DL28" s="29"/>
+      <c r="DM28" s="29"/>
+      <c r="DN28" s="29"/>
+      <c r="DO28" s="29"/>
+      <c r="DP28" s="29"/>
+      <c r="DQ28" s="29"/>
+      <c r="DR28" s="29"/>
+      <c r="DS28" s="29"/>
+      <c r="DT28" s="29"/>
+      <c r="DU28" s="29"/>
+      <c r="DV28" s="29"/>
+      <c r="DW28" s="29"/>
+      <c r="DX28" s="29"/>
+      <c r="DY28" s="29"/>
+      <c r="DZ28" s="29"/>
+      <c r="EA28" s="29"/>
+      <c r="EB28" s="29"/>
+      <c r="EC28" s="29"/>
+      <c r="ED28" s="29"/>
+      <c r="EE28" s="29"/>
+      <c r="EF28" s="29"/>
+      <c r="EG28" s="29"/>
+      <c r="EH28" s="29"/>
+      <c r="EI28" s="29"/>
+      <c r="EJ28" s="29"/>
+      <c r="EK28" s="29"/>
+      <c r="EL28" s="29"/>
+      <c r="EM28" s="29"/>
+      <c r="EN28" s="29"/>
+      <c r="EO28" s="29"/>
     </row>
     <row r="31" spans="1:145" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="CN31" s="1" t="s">
@@ -7027,6 +7034,300 @@
     </row>
   </sheetData>
   <mergeCells count="318">
+    <mergeCell ref="AO17:EO17"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="E2:E7"/>
+    <mergeCell ref="F2:F7"/>
+    <mergeCell ref="G2:G7"/>
+    <mergeCell ref="H2:H7"/>
+    <mergeCell ref="I2:I7"/>
+    <mergeCell ref="J2:J7"/>
+    <mergeCell ref="K2:K7"/>
+    <mergeCell ref="L2:L7"/>
+    <mergeCell ref="M2:M7"/>
+    <mergeCell ref="N2:N7"/>
+    <mergeCell ref="O2:O7"/>
+    <mergeCell ref="P2:P7"/>
+    <mergeCell ref="Q2:Q7"/>
+    <mergeCell ref="R2:R7"/>
+    <mergeCell ref="BM1:BO1"/>
+    <mergeCell ref="S2:S7"/>
+    <mergeCell ref="T2:T7"/>
+    <mergeCell ref="U2:U7"/>
+    <mergeCell ref="V2:V7"/>
+    <mergeCell ref="W2:W7"/>
+    <mergeCell ref="X2:X7"/>
+    <mergeCell ref="Y2:Y7"/>
+    <mergeCell ref="Z2:Z7"/>
+    <mergeCell ref="AA2:AA7"/>
+    <mergeCell ref="AB2:AB7"/>
+    <mergeCell ref="AC2:AC7"/>
+    <mergeCell ref="AD2:AD7"/>
+    <mergeCell ref="AE2:AE7"/>
+    <mergeCell ref="AF2:AF7"/>
+    <mergeCell ref="AG2:AG7"/>
+    <mergeCell ref="AH2:AH7"/>
+    <mergeCell ref="AI2:AI7"/>
+    <mergeCell ref="AJ2:AJ7"/>
+    <mergeCell ref="AK2:AK7"/>
+    <mergeCell ref="AL2:AL7"/>
+    <mergeCell ref="AM2:AM7"/>
+    <mergeCell ref="AN2:AN7"/>
+    <mergeCell ref="AO2:AO7"/>
+    <mergeCell ref="AP2:AP7"/>
+    <mergeCell ref="AQ2:AQ7"/>
+    <mergeCell ref="AR2:AR7"/>
+    <mergeCell ref="AS2:AS7"/>
+    <mergeCell ref="AT2:AT7"/>
+    <mergeCell ref="AU2:AU7"/>
+    <mergeCell ref="AV2:AV7"/>
+    <mergeCell ref="AW2:AW7"/>
+    <mergeCell ref="AX2:AX7"/>
+    <mergeCell ref="AY2:AY7"/>
+    <mergeCell ref="AZ2:AZ7"/>
+    <mergeCell ref="BA2:BA7"/>
+    <mergeCell ref="BB2:BB7"/>
+    <mergeCell ref="BC2:BC7"/>
+    <mergeCell ref="BD2:BD7"/>
+    <mergeCell ref="BE2:BE7"/>
+    <mergeCell ref="BF2:BF7"/>
+    <mergeCell ref="BG2:BG7"/>
+    <mergeCell ref="BH2:BH7"/>
+    <mergeCell ref="BI2:BI7"/>
+    <mergeCell ref="BJ2:BJ7"/>
+    <mergeCell ref="BK2:BK7"/>
+    <mergeCell ref="BL2:BL7"/>
+    <mergeCell ref="BM2:BM7"/>
+    <mergeCell ref="BN2:BN7"/>
+    <mergeCell ref="BO2:BO7"/>
+    <mergeCell ref="BP2:BP7"/>
+    <mergeCell ref="BQ2:BQ7"/>
+    <mergeCell ref="BR2:BR7"/>
+    <mergeCell ref="BS2:BS7"/>
+    <mergeCell ref="BT2:BT7"/>
+    <mergeCell ref="BU2:BU7"/>
+    <mergeCell ref="BV2:BV7"/>
+    <mergeCell ref="BW2:BW7"/>
+    <mergeCell ref="BX2:BX7"/>
+    <mergeCell ref="BY2:BY7"/>
+    <mergeCell ref="BZ2:BZ7"/>
+    <mergeCell ref="CA2:CA7"/>
+    <mergeCell ref="CB2:CB7"/>
+    <mergeCell ref="CC2:CC7"/>
+    <mergeCell ref="CD2:CD7"/>
+    <mergeCell ref="CE2:CE7"/>
+    <mergeCell ref="CF2:CF7"/>
+    <mergeCell ref="CG2:CG7"/>
+    <mergeCell ref="CH2:CH7"/>
+    <mergeCell ref="CI2:CI7"/>
+    <mergeCell ref="CJ2:CJ7"/>
+    <mergeCell ref="CK2:CK7"/>
+    <mergeCell ref="CL2:CL7"/>
+    <mergeCell ref="CM2:CM7"/>
+    <mergeCell ref="CN2:CN7"/>
+    <mergeCell ref="CO2:CO7"/>
+    <mergeCell ref="CP2:CP7"/>
+    <mergeCell ref="CQ2:CQ7"/>
+    <mergeCell ref="CR2:CR7"/>
+    <mergeCell ref="CS2:CS7"/>
+    <mergeCell ref="CT2:CT7"/>
+    <mergeCell ref="CU2:CU7"/>
+    <mergeCell ref="CV2:CV7"/>
+    <mergeCell ref="CW2:CW7"/>
+    <mergeCell ref="CX2:CX7"/>
+    <mergeCell ref="CY2:CY7"/>
+    <mergeCell ref="CZ2:CZ7"/>
+    <mergeCell ref="DA2:DA7"/>
+    <mergeCell ref="DB2:DB7"/>
+    <mergeCell ref="DC2:DC7"/>
+    <mergeCell ref="DD2:DD7"/>
+    <mergeCell ref="DE2:DE7"/>
+    <mergeCell ref="DF2:DF7"/>
+    <mergeCell ref="DG2:DG7"/>
+    <mergeCell ref="DH2:DH7"/>
+    <mergeCell ref="DI2:DI7"/>
+    <mergeCell ref="DJ2:DJ7"/>
+    <mergeCell ref="DK2:DK7"/>
+    <mergeCell ref="DL2:DL7"/>
+    <mergeCell ref="DM2:DM7"/>
+    <mergeCell ref="DN2:DN7"/>
+    <mergeCell ref="DO2:DO7"/>
+    <mergeCell ref="EF2:EF7"/>
+    <mergeCell ref="EG2:EG7"/>
+    <mergeCell ref="DP2:DP7"/>
+    <mergeCell ref="DQ2:DQ7"/>
+    <mergeCell ref="DR2:DR7"/>
+    <mergeCell ref="DS2:DS7"/>
+    <mergeCell ref="DT2:DT7"/>
+    <mergeCell ref="DU2:DU7"/>
+    <mergeCell ref="DV2:DV7"/>
+    <mergeCell ref="DW2:DW7"/>
+    <mergeCell ref="DX2:DX7"/>
+    <mergeCell ref="EH2:EH7"/>
+    <mergeCell ref="EI2:EI7"/>
+    <mergeCell ref="EJ2:EJ7"/>
+    <mergeCell ref="EK2:EK7"/>
+    <mergeCell ref="EL2:EL7"/>
+    <mergeCell ref="EM2:EM7"/>
+    <mergeCell ref="EN2:EN7"/>
+    <mergeCell ref="EO2:EO7"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="DY2:DY7"/>
+    <mergeCell ref="DZ2:DZ7"/>
+    <mergeCell ref="EA2:EA7"/>
+    <mergeCell ref="EB2:EB7"/>
+    <mergeCell ref="EC2:EC7"/>
+    <mergeCell ref="ED2:ED7"/>
+    <mergeCell ref="EE2:EE7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="S8:S9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="AE8:AE9"/>
+    <mergeCell ref="AF8:AF9"/>
+    <mergeCell ref="AG8:AG9"/>
+    <mergeCell ref="AH8:AH9"/>
+    <mergeCell ref="AI8:AI9"/>
+    <mergeCell ref="AJ8:AJ9"/>
+    <mergeCell ref="AK8:AK9"/>
+    <mergeCell ref="AL8:AL9"/>
+    <mergeCell ref="AM8:AM9"/>
+    <mergeCell ref="AN8:AN9"/>
+    <mergeCell ref="AO8:AO9"/>
+    <mergeCell ref="AP8:AP9"/>
+    <mergeCell ref="AQ8:AQ9"/>
+    <mergeCell ref="AR8:AR9"/>
+    <mergeCell ref="AS8:AS9"/>
+    <mergeCell ref="AT8:AT9"/>
+    <mergeCell ref="AU8:AU9"/>
+    <mergeCell ref="AV8:AV9"/>
+    <mergeCell ref="AW8:AW9"/>
+    <mergeCell ref="AX8:AX9"/>
+    <mergeCell ref="AY8:AY9"/>
+    <mergeCell ref="AZ8:AZ9"/>
+    <mergeCell ref="BA8:BA9"/>
+    <mergeCell ref="BB8:BB9"/>
+    <mergeCell ref="BC8:BC9"/>
+    <mergeCell ref="BD8:BD9"/>
+    <mergeCell ref="BE8:BE9"/>
+    <mergeCell ref="BF8:BF9"/>
+    <mergeCell ref="BG8:BG9"/>
+    <mergeCell ref="BH8:BH9"/>
+    <mergeCell ref="BI8:BI9"/>
+    <mergeCell ref="BJ8:BJ9"/>
+    <mergeCell ref="BK8:BK9"/>
+    <mergeCell ref="BL8:BL9"/>
+    <mergeCell ref="BM8:BM9"/>
+    <mergeCell ref="BN8:BN9"/>
+    <mergeCell ref="BO8:BO9"/>
+    <mergeCell ref="BP8:BP9"/>
+    <mergeCell ref="BQ8:BQ9"/>
+    <mergeCell ref="BR8:BR9"/>
+    <mergeCell ref="BS8:BS9"/>
+    <mergeCell ref="BT8:BT9"/>
+    <mergeCell ref="BU8:BU9"/>
+    <mergeCell ref="BV8:BV9"/>
+    <mergeCell ref="BW8:BW9"/>
+    <mergeCell ref="CN8:CN9"/>
+    <mergeCell ref="CO8:CO9"/>
+    <mergeCell ref="BX8:BX9"/>
+    <mergeCell ref="BY8:BY9"/>
+    <mergeCell ref="BZ8:BZ9"/>
+    <mergeCell ref="CA8:CA9"/>
+    <mergeCell ref="CB8:CB9"/>
+    <mergeCell ref="CC8:CC9"/>
+    <mergeCell ref="CD8:CD9"/>
+    <mergeCell ref="CE8:CE9"/>
+    <mergeCell ref="CF8:CF9"/>
+    <mergeCell ref="ED8:ED9"/>
+    <mergeCell ref="BH1:BL1"/>
+    <mergeCell ref="EE8:EE9"/>
+    <mergeCell ref="DD8:DD9"/>
+    <mergeCell ref="DE8:DE9"/>
+    <mergeCell ref="DF8:DF9"/>
+    <mergeCell ref="DG8:DG9"/>
+    <mergeCell ref="CP8:CP9"/>
+    <mergeCell ref="CQ8:CQ9"/>
+    <mergeCell ref="CR8:CR9"/>
+    <mergeCell ref="CS8:CS9"/>
+    <mergeCell ref="CT8:CT9"/>
+    <mergeCell ref="CU8:CU9"/>
+    <mergeCell ref="CV8:CV9"/>
+    <mergeCell ref="CW8:CW9"/>
+    <mergeCell ref="CX8:CX9"/>
+    <mergeCell ref="DC8:DC9"/>
+    <mergeCell ref="CG8:CG9"/>
+    <mergeCell ref="CH8:CH9"/>
+    <mergeCell ref="CI8:CI9"/>
+    <mergeCell ref="CJ8:CJ9"/>
+    <mergeCell ref="CK8:CK9"/>
+    <mergeCell ref="CL8:CL9"/>
+    <mergeCell ref="CM8:CM9"/>
+    <mergeCell ref="DA8:DA9"/>
+    <mergeCell ref="DB8:DB9"/>
+    <mergeCell ref="E28:EO28"/>
+    <mergeCell ref="AC1:AD1"/>
+    <mergeCell ref="AE1:AH1"/>
+    <mergeCell ref="AI1:AL1"/>
+    <mergeCell ref="AM1:AN1"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="AS1:AW1"/>
+    <mergeCell ref="AY1:BC1"/>
+    <mergeCell ref="BD1:BF1"/>
+    <mergeCell ref="EI8:EI9"/>
+    <mergeCell ref="EJ8:EJ9"/>
+    <mergeCell ref="EK8:EK9"/>
+    <mergeCell ref="EL8:EL9"/>
+    <mergeCell ref="EM8:EM9"/>
+    <mergeCell ref="EN8:EN9"/>
+    <mergeCell ref="EO8:EO9"/>
+    <mergeCell ref="EF8:EF9"/>
+    <mergeCell ref="EG8:EG9"/>
+    <mergeCell ref="DZ8:DZ9"/>
+    <mergeCell ref="EA8:EA9"/>
+    <mergeCell ref="EB8:EB9"/>
+    <mergeCell ref="EC8:EC9"/>
     <mergeCell ref="BZ1:CB1"/>
     <mergeCell ref="BQ1:BU1"/>
     <mergeCell ref="BV1:BX1"/>
@@ -7051,300 +7352,6 @@
     <mergeCell ref="DW8:DW9"/>
     <mergeCell ref="DX8:DX9"/>
     <mergeCell ref="DY8:DY9"/>
-    <mergeCell ref="DA8:DA9"/>
-    <mergeCell ref="DB8:DB9"/>
-    <mergeCell ref="E28:EO28"/>
-    <mergeCell ref="AC1:AD1"/>
-    <mergeCell ref="AE1:AH1"/>
-    <mergeCell ref="AI1:AL1"/>
-    <mergeCell ref="AM1:AN1"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="AS1:AW1"/>
-    <mergeCell ref="AY1:BC1"/>
-    <mergeCell ref="BD1:BF1"/>
-    <mergeCell ref="EI8:EI9"/>
-    <mergeCell ref="EJ8:EJ9"/>
-    <mergeCell ref="EK8:EK9"/>
-    <mergeCell ref="EL8:EL9"/>
-    <mergeCell ref="EM8:EM9"/>
-    <mergeCell ref="EN8:EN9"/>
-    <mergeCell ref="EO8:EO9"/>
-    <mergeCell ref="EF8:EF9"/>
-    <mergeCell ref="EG8:EG9"/>
-    <mergeCell ref="DZ8:DZ9"/>
-    <mergeCell ref="EA8:EA9"/>
-    <mergeCell ref="EB8:EB9"/>
-    <mergeCell ref="EC8:EC9"/>
-    <mergeCell ref="ED8:ED9"/>
-    <mergeCell ref="BH1:BL1"/>
-    <mergeCell ref="EE8:EE9"/>
-    <mergeCell ref="DD8:DD9"/>
-    <mergeCell ref="DE8:DE9"/>
-    <mergeCell ref="DF8:DF9"/>
-    <mergeCell ref="DG8:DG9"/>
-    <mergeCell ref="CP8:CP9"/>
-    <mergeCell ref="CQ8:CQ9"/>
-    <mergeCell ref="CR8:CR9"/>
-    <mergeCell ref="CS8:CS9"/>
-    <mergeCell ref="CT8:CT9"/>
-    <mergeCell ref="CU8:CU9"/>
-    <mergeCell ref="CV8:CV9"/>
-    <mergeCell ref="CW8:CW9"/>
-    <mergeCell ref="CX8:CX9"/>
-    <mergeCell ref="DC8:DC9"/>
-    <mergeCell ref="CG8:CG9"/>
-    <mergeCell ref="CH8:CH9"/>
-    <mergeCell ref="CI8:CI9"/>
-    <mergeCell ref="CJ8:CJ9"/>
-    <mergeCell ref="CK8:CK9"/>
-    <mergeCell ref="CL8:CL9"/>
-    <mergeCell ref="CM8:CM9"/>
-    <mergeCell ref="CN8:CN9"/>
-    <mergeCell ref="CO8:CO9"/>
-    <mergeCell ref="BX8:BX9"/>
-    <mergeCell ref="BY8:BY9"/>
-    <mergeCell ref="BZ8:BZ9"/>
-    <mergeCell ref="CA8:CA9"/>
-    <mergeCell ref="CB8:CB9"/>
-    <mergeCell ref="CC8:CC9"/>
-    <mergeCell ref="CD8:CD9"/>
-    <mergeCell ref="CE8:CE9"/>
-    <mergeCell ref="CF8:CF9"/>
-    <mergeCell ref="BO8:BO9"/>
-    <mergeCell ref="BP8:BP9"/>
-    <mergeCell ref="BQ8:BQ9"/>
-    <mergeCell ref="BR8:BR9"/>
-    <mergeCell ref="BS8:BS9"/>
-    <mergeCell ref="BT8:BT9"/>
-    <mergeCell ref="BU8:BU9"/>
-    <mergeCell ref="BV8:BV9"/>
-    <mergeCell ref="BW8:BW9"/>
-    <mergeCell ref="BF8:BF9"/>
-    <mergeCell ref="BG8:BG9"/>
-    <mergeCell ref="BH8:BH9"/>
-    <mergeCell ref="BI8:BI9"/>
-    <mergeCell ref="BJ8:BJ9"/>
-    <mergeCell ref="BK8:BK9"/>
-    <mergeCell ref="BL8:BL9"/>
-    <mergeCell ref="BM8:BM9"/>
-    <mergeCell ref="BN8:BN9"/>
-    <mergeCell ref="AW8:AW9"/>
-    <mergeCell ref="AX8:AX9"/>
-    <mergeCell ref="AY8:AY9"/>
-    <mergeCell ref="AZ8:AZ9"/>
-    <mergeCell ref="BA8:BA9"/>
-    <mergeCell ref="BB8:BB9"/>
-    <mergeCell ref="BC8:BC9"/>
-    <mergeCell ref="BD8:BD9"/>
-    <mergeCell ref="BE8:BE9"/>
-    <mergeCell ref="AN8:AN9"/>
-    <mergeCell ref="AO8:AO9"/>
-    <mergeCell ref="AP8:AP9"/>
-    <mergeCell ref="AQ8:AQ9"/>
-    <mergeCell ref="AR8:AR9"/>
-    <mergeCell ref="AS8:AS9"/>
-    <mergeCell ref="AT8:AT9"/>
-    <mergeCell ref="AU8:AU9"/>
-    <mergeCell ref="AV8:AV9"/>
-    <mergeCell ref="AE8:AE9"/>
-    <mergeCell ref="AF8:AF9"/>
-    <mergeCell ref="AG8:AG9"/>
-    <mergeCell ref="AH8:AH9"/>
-    <mergeCell ref="AI8:AI9"/>
-    <mergeCell ref="AJ8:AJ9"/>
-    <mergeCell ref="AK8:AK9"/>
-    <mergeCell ref="AL8:AL9"/>
-    <mergeCell ref="AM8:AM9"/>
-    <mergeCell ref="V8:V9"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="Y8:Y9"/>
-    <mergeCell ref="Z8:Z9"/>
-    <mergeCell ref="AA8:AA9"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="U8:U9"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="EH2:EH7"/>
-    <mergeCell ref="EI2:EI7"/>
-    <mergeCell ref="EJ2:EJ7"/>
-    <mergeCell ref="EK2:EK7"/>
-    <mergeCell ref="EL2:EL7"/>
-    <mergeCell ref="EM2:EM7"/>
-    <mergeCell ref="EN2:EN7"/>
-    <mergeCell ref="EO2:EO7"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="DY2:DY7"/>
-    <mergeCell ref="DZ2:DZ7"/>
-    <mergeCell ref="EA2:EA7"/>
-    <mergeCell ref="EB2:EB7"/>
-    <mergeCell ref="EC2:EC7"/>
-    <mergeCell ref="ED2:ED7"/>
-    <mergeCell ref="EE2:EE7"/>
-    <mergeCell ref="DN2:DN7"/>
-    <mergeCell ref="DO2:DO7"/>
-    <mergeCell ref="EF2:EF7"/>
-    <mergeCell ref="EG2:EG7"/>
-    <mergeCell ref="DP2:DP7"/>
-    <mergeCell ref="DQ2:DQ7"/>
-    <mergeCell ref="DR2:DR7"/>
-    <mergeCell ref="DS2:DS7"/>
-    <mergeCell ref="DT2:DT7"/>
-    <mergeCell ref="DU2:DU7"/>
-    <mergeCell ref="DV2:DV7"/>
-    <mergeCell ref="DW2:DW7"/>
-    <mergeCell ref="DX2:DX7"/>
-    <mergeCell ref="DE2:DE7"/>
-    <mergeCell ref="DF2:DF7"/>
-    <mergeCell ref="DG2:DG7"/>
-    <mergeCell ref="DH2:DH7"/>
-    <mergeCell ref="DI2:DI7"/>
-    <mergeCell ref="DJ2:DJ7"/>
-    <mergeCell ref="DK2:DK7"/>
-    <mergeCell ref="DL2:DL7"/>
-    <mergeCell ref="DM2:DM7"/>
-    <mergeCell ref="CV2:CV7"/>
-    <mergeCell ref="CW2:CW7"/>
-    <mergeCell ref="CX2:CX7"/>
-    <mergeCell ref="CY2:CY7"/>
-    <mergeCell ref="CZ2:CZ7"/>
-    <mergeCell ref="DA2:DA7"/>
-    <mergeCell ref="DB2:DB7"/>
-    <mergeCell ref="DC2:DC7"/>
-    <mergeCell ref="DD2:DD7"/>
-    <mergeCell ref="CM2:CM7"/>
-    <mergeCell ref="CN2:CN7"/>
-    <mergeCell ref="CO2:CO7"/>
-    <mergeCell ref="CP2:CP7"/>
-    <mergeCell ref="CQ2:CQ7"/>
-    <mergeCell ref="CR2:CR7"/>
-    <mergeCell ref="CS2:CS7"/>
-    <mergeCell ref="CT2:CT7"/>
-    <mergeCell ref="CU2:CU7"/>
-    <mergeCell ref="CD2:CD7"/>
-    <mergeCell ref="CE2:CE7"/>
-    <mergeCell ref="CF2:CF7"/>
-    <mergeCell ref="CG2:CG7"/>
-    <mergeCell ref="CH2:CH7"/>
-    <mergeCell ref="CI2:CI7"/>
-    <mergeCell ref="CJ2:CJ7"/>
-    <mergeCell ref="CK2:CK7"/>
-    <mergeCell ref="CL2:CL7"/>
-    <mergeCell ref="BU2:BU7"/>
-    <mergeCell ref="BV2:BV7"/>
-    <mergeCell ref="BW2:BW7"/>
-    <mergeCell ref="BX2:BX7"/>
-    <mergeCell ref="BY2:BY7"/>
-    <mergeCell ref="BZ2:BZ7"/>
-    <mergeCell ref="CA2:CA7"/>
-    <mergeCell ref="CB2:CB7"/>
-    <mergeCell ref="CC2:CC7"/>
-    <mergeCell ref="BL2:BL7"/>
-    <mergeCell ref="BM2:BM7"/>
-    <mergeCell ref="BN2:BN7"/>
-    <mergeCell ref="BO2:BO7"/>
-    <mergeCell ref="BP2:BP7"/>
-    <mergeCell ref="BQ2:BQ7"/>
-    <mergeCell ref="BR2:BR7"/>
-    <mergeCell ref="BS2:BS7"/>
-    <mergeCell ref="BT2:BT7"/>
-    <mergeCell ref="BC2:BC7"/>
-    <mergeCell ref="BD2:BD7"/>
-    <mergeCell ref="BE2:BE7"/>
-    <mergeCell ref="BF2:BF7"/>
-    <mergeCell ref="BG2:BG7"/>
-    <mergeCell ref="BH2:BH7"/>
-    <mergeCell ref="BI2:BI7"/>
-    <mergeCell ref="BJ2:BJ7"/>
-    <mergeCell ref="BK2:BK7"/>
-    <mergeCell ref="AT2:AT7"/>
-    <mergeCell ref="AU2:AU7"/>
-    <mergeCell ref="AV2:AV7"/>
-    <mergeCell ref="AW2:AW7"/>
-    <mergeCell ref="AX2:AX7"/>
-    <mergeCell ref="AY2:AY7"/>
-    <mergeCell ref="AZ2:AZ7"/>
-    <mergeCell ref="BA2:BA7"/>
-    <mergeCell ref="BB2:BB7"/>
-    <mergeCell ref="AK2:AK7"/>
-    <mergeCell ref="AL2:AL7"/>
-    <mergeCell ref="AM2:AM7"/>
-    <mergeCell ref="AN2:AN7"/>
-    <mergeCell ref="AO2:AO7"/>
-    <mergeCell ref="AP2:AP7"/>
-    <mergeCell ref="AQ2:AQ7"/>
-    <mergeCell ref="AR2:AR7"/>
-    <mergeCell ref="AS2:AS7"/>
-    <mergeCell ref="AB2:AB7"/>
-    <mergeCell ref="AC2:AC7"/>
-    <mergeCell ref="AD2:AD7"/>
-    <mergeCell ref="AE2:AE7"/>
-    <mergeCell ref="AF2:AF7"/>
-    <mergeCell ref="AG2:AG7"/>
-    <mergeCell ref="AH2:AH7"/>
-    <mergeCell ref="AI2:AI7"/>
-    <mergeCell ref="AJ2:AJ7"/>
-    <mergeCell ref="S2:S7"/>
-    <mergeCell ref="T2:T7"/>
-    <mergeCell ref="U2:U7"/>
-    <mergeCell ref="V2:V7"/>
-    <mergeCell ref="W2:W7"/>
-    <mergeCell ref="X2:X7"/>
-    <mergeCell ref="Y2:Y7"/>
-    <mergeCell ref="Z2:Z7"/>
-    <mergeCell ref="AA2:AA7"/>
-    <mergeCell ref="AO17:EO17"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:D2"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="E2:E7"/>
-    <mergeCell ref="F2:F7"/>
-    <mergeCell ref="G2:G7"/>
-    <mergeCell ref="H2:H7"/>
-    <mergeCell ref="I2:I7"/>
-    <mergeCell ref="J2:J7"/>
-    <mergeCell ref="K2:K7"/>
-    <mergeCell ref="L2:L7"/>
-    <mergeCell ref="M2:M7"/>
-    <mergeCell ref="N2:N7"/>
-    <mergeCell ref="O2:O7"/>
-    <mergeCell ref="P2:P7"/>
-    <mergeCell ref="Q2:Q7"/>
-    <mergeCell ref="R2:R7"/>
-    <mergeCell ref="BM1:BO1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0"/>

</xml_diff>